<commit_message>
fix: Add missing find_new_feature_column and get_brd_data_for_new_feature_task methods to BrdMatcher
</commit_message>
<xml_diff>
--- a/asana_generator_app/resources/Template.xlsx
+++ b/asana_generator_app/resources/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sakthivelprabakaran/Documents/Prabakaran/ASANA/ASANA_Dashboard/asana_generator_app/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sakthimx\Desktop\ASANA_Dashboard\asana_generator_app\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597780BA-4D05-FA4C-A47F-D23DBDA2E2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109D34C8-BB9E-41E0-AB96-8FF846F700B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="640" windowWidth="28040" windowHeight="16280" firstSheet="2" activeTab="8" xr2:uid="{65F45C9F-47C9-5D42-9768-363B1ABC41FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="11" activeTab="15" xr2:uid="{65F45C9F-47C9-5D42-9768-363B1ABC41FB}"/>
   </bookViews>
   <sheets>
     <sheet name="P0" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,7 @@
     <sheet name="HWR Search" sheetId="14" r:id="rId13"/>
     <sheet name="Keyboard_canvas" sheetId="15" r:id="rId14"/>
     <sheet name="Q&amp;A" sheetId="16" r:id="rId15"/>
+    <sheet name="Dark_mode" sheetId="17" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="265">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -797,13 +798,58 @@
   </si>
   <si>
     <t>OOBE 1X</t>
+  </si>
+  <si>
+    <t>search in home "digital" [Medium occurance of selected word in book] - having collections</t>
+  </si>
+  <si>
+    <t>Canvas write" K "letter to predictive letter</t>
+  </si>
+  <si>
+    <t>Canvas write "K" letter to search suggestion</t>
+  </si>
+  <si>
+    <t>Canvas write "Kindle" letter to predictive</t>
+  </si>
+  <si>
+    <t>Canvas write "Kindle" letter to search suggestion</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Two Step Verification' page from password page</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Verify Account' page from password page.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Create a New Account: Country selector' screen from registration screen.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load Goodreads sign-in / Sign-up' page from 'Get the Kindle App' screen</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load Prime 'Upsell' page from 'Get the Kindle App' screen</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load KU 'Upsell' page from 'Get the Kindle App' screen</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load Audible 'Upsell' page from 'Get the Kindle App' screen.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Create New Account' confirmation dialog from goodreads page.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Sign In to GoodReads' page from goodreads page.</t>
+  </si>
+  <si>
+    <t>Rossini,Seabreeze,Calvados,Pisco</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -887,7 +933,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -953,6 +999,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -971,9 +1020,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1011,7 +1060,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1117,7 +1166,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1259,7 +1308,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1268,7 +1317,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE18BECF-6DD2-2040-96C2-5A669DEC5545}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="39.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -1277,7 +1326,7 @@
     <col min="5" max="5" width="6.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1297,7 +1346,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="17.5">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1311,7 +1360,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="17.5">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1325,7 +1374,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="29">
       <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
@@ -1339,7 +1388,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="17.5">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -1361,9 +1410,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79727740-68CD-9542-B80B-1E27161C7735}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1391,7 +1440,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7FB816-C3BB-A141-B123-3CDD37829D2C}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1400,7 +1449,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDD20E5F-03C6-A74F-90C7-31AA338BEEE2}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="55.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -1408,7 +1457,7 @@
     <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1428,7 +1477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="24" t="s">
         <v>24</v>
       </c>
@@ -1442,7 +1491,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="24" t="s">
         <v>25</v>
       </c>
@@ -1456,7 +1505,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="24" t="s">
         <v>26</v>
       </c>
@@ -1470,7 +1519,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="24" t="s">
         <v>217</v>
       </c>
@@ -1484,7 +1533,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="24" t="s">
         <v>218</v>
       </c>
@@ -1498,7 +1547,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
         <v>24</v>
       </c>
@@ -1512,7 +1561,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
         <v>25</v>
       </c>
@@ -1526,7 +1575,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
         <v>26</v>
       </c>
@@ -1540,7 +1589,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
         <v>217</v>
       </c>
@@ -1554,7 +1603,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
         <v>218</v>
       </c>
@@ -1576,14 +1625,14 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97633E95-5463-BE46-889E-C8CD75E087A0}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="56.33203125" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1603,7 +1652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="9" t="s">
         <v>220</v>
       </c>
@@ -1617,7 +1666,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
         <v>221</v>
       </c>
@@ -1631,7 +1680,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
         <v>222</v>
       </c>
@@ -1645,7 +1694,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="31">
       <c r="A5" s="9" t="s">
         <v>223</v>
       </c>
@@ -1659,7 +1708,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
         <v>224</v>
       </c>
@@ -1673,7 +1722,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="31">
       <c r="A7" s="9" t="s">
         <v>225</v>
       </c>
@@ -1687,7 +1736,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="31">
       <c r="A8" s="9" t="s">
         <v>226</v>
       </c>
@@ -1701,7 +1750,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
         <v>227</v>
       </c>
@@ -1715,7 +1764,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="31">
       <c r="A10" s="9" t="s">
         <v>228</v>
       </c>
@@ -1729,7 +1778,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
         <v>229</v>
       </c>
@@ -1743,7 +1792,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
         <v>230</v>
       </c>
@@ -1757,7 +1806,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
         <v>231</v>
       </c>
@@ -1771,7 +1820,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="9" t="s">
         <v>232</v>
       </c>
@@ -1785,7 +1834,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="31">
       <c r="A15" s="9" t="s">
         <v>233</v>
       </c>
@@ -1799,7 +1848,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="31">
       <c r="A16" s="9" t="s">
         <v>234</v>
       </c>
@@ -1813,7 +1862,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="31">
       <c r="A17" s="9" t="s">
         <v>235</v>
       </c>
@@ -1827,7 +1876,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="31">
       <c r="A18" s="9" t="s">
         <v>236</v>
       </c>
@@ -1841,7 +1890,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="31">
       <c r="A19" s="8" t="s">
         <v>237</v>
       </c>
@@ -1863,7 +1912,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1AA77A7-5CD2-4A4E-B4AB-1458D30C67D9}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -1871,7 +1920,7 @@
     <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1891,7 +1940,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="8" t="s">
         <v>210</v>
       </c>
@@ -1905,7 +1954,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
         <v>211</v>
       </c>
@@ -1919,7 +1968,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
         <v>212</v>
       </c>
@@ -1933,7 +1982,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
         <v>213</v>
       </c>
@@ -1947,7 +1996,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="8" t="s">
         <v>214</v>
       </c>
@@ -1961,7 +2010,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
         <v>215</v>
       </c>
@@ -1975,7 +2024,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
         <v>216</v>
       </c>
@@ -1989,7 +2038,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
         <v>210</v>
       </c>
@@ -2003,7 +2052,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
         <v>211</v>
       </c>
@@ -2017,7 +2066,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
         <v>212</v>
       </c>
@@ -2039,14 +2088,14 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72501A7C-CDA9-A44E-9BDB-DD2473AB4D78}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="56.33203125" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2066,7 +2115,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="9" t="s">
         <v>241</v>
       </c>
@@ -2080,7 +2129,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
         <v>242</v>
       </c>
@@ -2094,7 +2143,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
         <v>243</v>
       </c>
@@ -2108,7 +2157,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
         <v>244</v>
       </c>
@@ -2122,7 +2171,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
         <v>245</v>
       </c>
@@ -2136,7 +2185,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
         <v>241</v>
       </c>
@@ -2150,7 +2199,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
         <v>242</v>
       </c>
@@ -2164,7 +2213,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
         <v>243</v>
       </c>
@@ -2178,7 +2227,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
         <v>244</v>
       </c>
@@ -2192,7 +2241,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
         <v>245</v>
       </c>
@@ -2203,6 +2252,746 @@
         <v>239</v>
       </c>
       <c r="E11" s="12">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{151D4084-A461-4CDA-9C30-D3B244C2EA06}">
+  <dimension ref="A1:F65"/>
+  <sheetFormatPr defaultRowHeight="15.5"/>
+  <cols>
+    <col min="1" max="1" width="52.58203125" customWidth="1"/>
+    <col min="2" max="2" width="27.9140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.58203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.9140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="31">
+      <c r="A2" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E2" s="25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="31">
+      <c r="A3" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E3" s="25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="46.5">
+      <c r="A4" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" t="s">
+        <v>264</v>
+      </c>
+      <c r="E4" s="25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="31">
+      <c r="A5" s="25" t="s">
+        <v>160</v>
+      </c>
+      <c r="D5" t="s">
+        <v>264</v>
+      </c>
+      <c r="E5" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="31">
+      <c r="A6" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" t="s">
+        <v>264</v>
+      </c>
+      <c r="E6" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="46.5">
+      <c r="A7" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="D7" t="s">
+        <v>264</v>
+      </c>
+      <c r="E7" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="46.5">
+      <c r="A8" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
+        <v>264</v>
+      </c>
+      <c r="E8" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="46.5">
+      <c r="A9" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="D9" t="s">
+        <v>264</v>
+      </c>
+      <c r="E9" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="46.5">
+      <c r="A10" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="D10" t="s">
+        <v>264</v>
+      </c>
+      <c r="E10" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="62">
+      <c r="A11" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="D11" t="s">
+        <v>264</v>
+      </c>
+      <c r="E11" s="25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="31">
+      <c r="A12" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="D12" t="s">
+        <v>264</v>
+      </c>
+      <c r="E12" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" t="s">
+        <v>238</v>
+      </c>
+      <c r="E13" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="D14" t="s">
+        <v>238</v>
+      </c>
+      <c r="E14" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="46.5">
+      <c r="A15" s="25" t="s">
+        <v>251</v>
+      </c>
+      <c r="D15" t="s">
+        <v>238</v>
+      </c>
+      <c r="E15" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="46.5">
+      <c r="A16" s="25" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" t="s">
+        <v>238</v>
+      </c>
+      <c r="E16" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="46.5">
+      <c r="A17" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="D17" t="s">
+        <v>238</v>
+      </c>
+      <c r="E17" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="46.5">
+      <c r="A18" s="25" t="s">
+        <v>254</v>
+      </c>
+      <c r="D18" t="s">
+        <v>238</v>
+      </c>
+      <c r="E18" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="31">
+      <c r="A19" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="D19" t="s">
+        <v>238</v>
+      </c>
+      <c r="E19" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="D20" t="s">
+        <v>238</v>
+      </c>
+      <c r="E20" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="D21" t="s">
+        <v>238</v>
+      </c>
+      <c r="E21" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="62">
+      <c r="A22" s="25" t="s">
+        <v>220</v>
+      </c>
+      <c r="D22" t="s">
+        <v>238</v>
+      </c>
+      <c r="E22" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="62">
+      <c r="A23" s="25" t="s">
+        <v>221</v>
+      </c>
+      <c r="D23" t="s">
+        <v>238</v>
+      </c>
+      <c r="E23" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="62">
+      <c r="A24" s="25" t="s">
+        <v>222</v>
+      </c>
+      <c r="D24" t="s">
+        <v>238</v>
+      </c>
+      <c r="E24" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="77.5">
+      <c r="A25" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="D25" t="s">
+        <v>238</v>
+      </c>
+      <c r="E25" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="46.5">
+      <c r="A26" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="D26" t="s">
+        <v>238</v>
+      </c>
+      <c r="E26" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="77.5">
+      <c r="A27" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="D27" t="s">
+        <v>238</v>
+      </c>
+      <c r="E27" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="77.5">
+      <c r="A28" s="25" t="s">
+        <v>226</v>
+      </c>
+      <c r="D28" t="s">
+        <v>238</v>
+      </c>
+      <c r="E28" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="62">
+      <c r="A29" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="D29" t="s">
+        <v>238</v>
+      </c>
+      <c r="E29" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="77.5">
+      <c r="A30" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="D30" t="s">
+        <v>238</v>
+      </c>
+      <c r="E30" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="31">
+      <c r="A31" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="D31" t="s">
+        <v>238</v>
+      </c>
+      <c r="E31" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="31">
+      <c r="A32" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="D32" t="s">
+        <v>238</v>
+      </c>
+      <c r="E32" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="46.5">
+      <c r="A33" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="D33" t="s">
+        <v>238</v>
+      </c>
+      <c r="E33" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="46.5">
+      <c r="A34" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="D34" t="s">
+        <v>238</v>
+      </c>
+      <c r="E34" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="62">
+      <c r="A35" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="D35" t="s">
+        <v>238</v>
+      </c>
+      <c r="E35" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="62">
+      <c r="A36" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="D36" t="s">
+        <v>238</v>
+      </c>
+      <c r="E36" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="77.5">
+      <c r="A37" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="D37" t="s">
+        <v>238</v>
+      </c>
+      <c r="E37" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="62">
+      <c r="A38" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="D38" t="s">
+        <v>238</v>
+      </c>
+      <c r="E38" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="93">
+      <c r="A39" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="D39" t="s">
+        <v>238</v>
+      </c>
+      <c r="E39" s="25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="93">
+      <c r="A40" s="25" t="s">
+        <v>178</v>
+      </c>
+      <c r="D40" t="s">
+        <v>264</v>
+      </c>
+      <c r="E40" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="77.5">
+      <c r="A41" s="25" t="s">
+        <v>255</v>
+      </c>
+      <c r="D41" t="s">
+        <v>264</v>
+      </c>
+      <c r="E41" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="93">
+      <c r="A42" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="D42" t="s">
+        <v>264</v>
+      </c>
+      <c r="E42" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="62">
+      <c r="A43" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="D43" t="s">
+        <v>264</v>
+      </c>
+      <c r="E43" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="77.5">
+      <c r="A44" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="D44" t="s">
+        <v>264</v>
+      </c>
+      <c r="E44" s="25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="93">
+      <c r="A45" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="D45" t="s">
+        <v>264</v>
+      </c>
+      <c r="E45" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="93">
+      <c r="A46" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="D46" t="s">
+        <v>264</v>
+      </c>
+      <c r="E46" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="77.5">
+      <c r="A47" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="D47" t="s">
+        <v>264</v>
+      </c>
+      <c r="E47" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="77.5">
+      <c r="A48" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="D48" t="s">
+        <v>264</v>
+      </c>
+      <c r="E48" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="77.5">
+      <c r="A49" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="D49" t="s">
+        <v>264</v>
+      </c>
+      <c r="E49" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="62">
+      <c r="A50" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="D50" t="s">
+        <v>264</v>
+      </c>
+      <c r="E50" s="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="93">
+      <c r="A51" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="D51" t="s">
+        <v>264</v>
+      </c>
+      <c r="E51" s="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="93">
+      <c r="A52" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="D52" t="s">
+        <v>264</v>
+      </c>
+      <c r="E52" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="108.5">
+      <c r="A53" s="25" t="s">
+        <v>190</v>
+      </c>
+      <c r="D53" t="s">
+        <v>264</v>
+      </c>
+      <c r="E53" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="108.5">
+      <c r="A54" s="25" t="s">
+        <v>262</v>
+      </c>
+      <c r="D54" t="s">
+        <v>264</v>
+      </c>
+      <c r="E54" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="93">
+      <c r="A55" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="D55" t="s">
+        <v>264</v>
+      </c>
+      <c r="E55" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="108.5">
+      <c r="A56" s="25" t="s">
+        <v>193</v>
+      </c>
+      <c r="D56" t="s">
+        <v>264</v>
+      </c>
+      <c r="E56" s="25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="93">
+      <c r="A57" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="D57" t="s">
+        <v>264</v>
+      </c>
+      <c r="E57" s="25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="62">
+      <c r="A58" s="25" t="s">
+        <v>195</v>
+      </c>
+      <c r="D58" t="s">
+        <v>264</v>
+      </c>
+      <c r="E58" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="77.5">
+      <c r="A59" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="D59" t="s">
+        <v>264</v>
+      </c>
+      <c r="E59" s="25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="62">
+      <c r="A60" s="25" t="s">
+        <v>202</v>
+      </c>
+      <c r="D60" t="s">
+        <v>264</v>
+      </c>
+      <c r="E60" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="77.5">
+      <c r="A61" s="25" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" t="s">
+        <v>264</v>
+      </c>
+      <c r="E61" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="62">
+      <c r="A62" s="25" t="s">
+        <v>204</v>
+      </c>
+      <c r="D62" t="s">
+        <v>264</v>
+      </c>
+      <c r="E62" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="77.5">
+      <c r="A63" s="25" t="s">
+        <v>205</v>
+      </c>
+      <c r="D63" t="s">
+        <v>264</v>
+      </c>
+      <c r="E63" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="62">
+      <c r="A64" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="D64" t="s">
+        <v>264</v>
+      </c>
+      <c r="E64" s="25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="62">
+      <c r="A65" s="25" t="s">
+        <v>207</v>
+      </c>
+      <c r="D65" t="s">
+        <v>264</v>
+      </c>
+      <c r="E65" s="25">
         <v>30</v>
       </c>
     </row>
@@ -2214,7 +3003,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3C4C592-45AD-3F47-8199-72C481C3BD16}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -2222,7 +3011,7 @@
     <col min="4" max="4" width="32.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2242,7 +3031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="46.5">
       <c r="A2" s="8" t="s">
         <v>65</v>
       </c>
@@ -2256,7 +3045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="46.5">
       <c r="A3" s="8" t="s">
         <v>66</v>
       </c>
@@ -2270,7 +3059,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="46.5">
       <c r="A4" s="8" t="s">
         <v>67</v>
       </c>
@@ -2284,7 +3073,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="46.5">
       <c r="A5" s="8" t="s">
         <v>68</v>
       </c>
@@ -2298,7 +3087,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="46.5">
       <c r="A6" s="8" t="s">
         <v>69</v>
       </c>
@@ -2312,7 +3101,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="46.5">
       <c r="A7" s="8" t="s">
         <v>70</v>
       </c>
@@ -2326,7 +3115,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="46.5">
       <c r="A8" s="8" t="s">
         <v>71</v>
       </c>
@@ -2340,7 +3129,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="46.5">
       <c r="A9" s="8" t="s">
         <v>72</v>
       </c>
@@ -2362,7 +3151,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8414CF9-37A4-564E-A42E-4E0D99ADC213}">
   <dimension ref="A1:F56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="87.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -2370,7 +3159,7 @@
     <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2390,7 +3179,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
         <v>13</v>
       </c>
@@ -2404,7 +3193,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
         <v>14</v>
       </c>
@@ -2418,7 +3207,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
@@ -2432,7 +3221,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="7" t="s">
         <v>16</v>
       </c>
@@ -2446,7 +3235,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="31">
       <c r="A6" s="6" t="s">
         <v>17</v>
       </c>
@@ -2460,7 +3249,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
         <v>18</v>
       </c>
@@ -2474,7 +3263,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
         <v>19</v>
       </c>
@@ -2488,7 +3277,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
         <v>20</v>
       </c>
@@ -2502,7 +3291,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
         <v>21</v>
       </c>
@@ -2516,7 +3305,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
         <v>22</v>
       </c>
@@ -2530,7 +3319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="8" t="s">
         <v>23</v>
       </c>
@@ -2544,7 +3333,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="8" t="s">
         <v>24</v>
       </c>
@@ -2558,7 +3347,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="8" t="s">
         <v>25</v>
       </c>
@@ -2572,7 +3361,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="8" t="s">
         <v>26</v>
       </c>
@@ -2586,7 +3375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" s="9" t="s">
         <v>27</v>
       </c>
@@ -2600,7 +3389,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="9" t="s">
         <v>28</v>
       </c>
@@ -2614,7 +3403,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="31">
       <c r="A18" s="10" t="s">
         <v>29</v>
       </c>
@@ -2628,7 +3417,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5">
       <c r="A19" s="8" t="s">
         <v>30</v>
       </c>
@@ -2642,7 +3431,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5">
       <c r="A20" s="8" t="s">
         <v>31</v>
       </c>
@@ -2656,7 +3445,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5">
       <c r="A21" s="8" t="s">
         <v>32</v>
       </c>
@@ -2670,7 +3459,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5">
       <c r="A22" s="9" t="s">
         <v>33</v>
       </c>
@@ -2684,7 +3473,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5">
       <c r="A23" s="9" t="s">
         <v>34</v>
       </c>
@@ -2698,7 +3487,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" ht="31">
       <c r="A24" s="8" t="s">
         <v>35</v>
       </c>
@@ -2712,7 +3501,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5">
       <c r="A25" s="8" t="s">
         <v>36</v>
       </c>
@@ -2726,7 +3515,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5">
       <c r="A26" s="8" t="s">
         <v>37</v>
       </c>
@@ -2740,7 +3529,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5">
       <c r="A27" s="8" t="s">
         <v>38</v>
       </c>
@@ -2754,7 +3543,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5">
       <c r="A28" s="8" t="s">
         <v>39</v>
       </c>
@@ -2768,7 +3557,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5">
       <c r="A29" s="8" t="s">
         <v>40</v>
       </c>
@@ -2782,7 +3571,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5">
       <c r="A30" s="8" t="s">
         <v>41</v>
       </c>
@@ -2796,7 +3585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5">
       <c r="A31" s="8" t="s">
         <v>42</v>
       </c>
@@ -2810,7 +3599,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5">
       <c r="A32" s="8" t="s">
         <v>43</v>
       </c>
@@ -2824,7 +3613,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -2838,7 +3627,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5">
       <c r="A34" s="8" t="s">
         <v>45</v>
       </c>
@@ -2852,7 +3641,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5">
       <c r="A35" s="8" t="s">
         <v>46</v>
       </c>
@@ -2866,7 +3655,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -2880,7 +3669,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -2894,7 +3683,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -2908,7 +3697,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5">
       <c r="A39" s="8" t="s">
         <v>50</v>
       </c>
@@ -2922,7 +3711,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5">
       <c r="A40" s="8" t="s">
         <v>51</v>
       </c>
@@ -2936,7 +3725,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5">
       <c r="A41" s="8" t="s">
         <v>52</v>
       </c>
@@ -2950,7 +3739,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5">
       <c r="A42" s="8" t="s">
         <v>53</v>
       </c>
@@ -2964,7 +3753,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5">
       <c r="A43" s="8" t="s">
         <v>54</v>
       </c>
@@ -2978,7 +3767,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5">
       <c r="A44" s="9" t="s">
         <v>55</v>
       </c>
@@ -2992,7 +3781,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5">
       <c r="A45" s="8" t="s">
         <v>56</v>
       </c>
@@ -3006,7 +3795,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5">
       <c r="A46" s="8" t="s">
         <v>57</v>
       </c>
@@ -3020,7 +3809,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5">
       <c r="A47" s="9" t="s">
         <v>58</v>
       </c>
@@ -3034,7 +3823,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5">
       <c r="A48" s="8" t="s">
         <v>59</v>
       </c>
@@ -3048,7 +3837,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5">
       <c r="A49" s="8" t="s">
         <v>20</v>
       </c>
@@ -3062,7 +3851,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5">
       <c r="A50" s="8" t="s">
         <v>22</v>
       </c>
@@ -3076,7 +3865,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5">
       <c r="A51" s="8" t="s">
         <v>56</v>
       </c>
@@ -3090,7 +3879,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5">
       <c r="A52" s="8" t="s">
         <v>60</v>
       </c>
@@ -3104,7 +3893,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5">
       <c r="A53" s="8" t="s">
         <v>20</v>
       </c>
@@ -3118,7 +3907,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5">
       <c r="A54" s="8" t="s">
         <v>22</v>
       </c>
@@ -3132,7 +3921,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5">
       <c r="A55" s="8" t="s">
         <v>56</v>
       </c>
@@ -3146,7 +3935,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5">
       <c r="A56" s="8" t="s">
         <v>60</v>
       </c>
@@ -3169,7 +3958,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C45492B4-6712-F94F-B4BF-B31212E07AA7}">
   <dimension ref="A1:F57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="112" style="17" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -3177,7 +3966,7 @@
     <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -3197,7 +3986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="14" t="s">
         <v>74</v>
       </c>
@@ -3211,7 +4000,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="15" t="s">
         <v>75</v>
       </c>
@@ -3225,7 +4014,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="14" t="s">
         <v>76</v>
       </c>
@@ -3239,7 +4028,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="14" t="s">
         <v>77</v>
       </c>
@@ -3253,7 +4042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="14" t="s">
         <v>78</v>
       </c>
@@ -3267,7 +4056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="14" t="s">
         <v>79</v>
       </c>
@@ -3281,7 +4070,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="14" t="s">
         <v>80</v>
       </c>
@@ -3295,7 +4084,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="14" t="s">
         <v>81</v>
       </c>
@@ -3309,7 +4098,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="14" t="s">
         <v>82</v>
       </c>
@@ -3323,7 +4112,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="14" t="s">
         <v>83</v>
       </c>
@@ -3337,7 +4126,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="14" t="s">
         <v>84</v>
       </c>
@@ -3351,7 +4140,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="14" t="s">
         <v>85</v>
       </c>
@@ -3365,7 +4154,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="14" t="s">
         <v>86</v>
       </c>
@@ -3379,7 +4168,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="16" t="s">
         <v>87</v>
       </c>
@@ -3393,7 +4182,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" s="16" t="s">
         <v>88</v>
       </c>
@@ -3407,7 +4196,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="16" t="s">
         <v>89</v>
       </c>
@@ -3421,7 +4210,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5">
       <c r="A18" s="11" t="s">
         <v>90</v>
       </c>
@@ -3435,7 +4224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5">
       <c r="A19" s="9" t="s">
         <v>91</v>
       </c>
@@ -3449,7 +4238,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5">
       <c r="A20" s="9" t="s">
         <v>92</v>
       </c>
@@ -3463,7 +4252,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5">
       <c r="A21" s="9" t="s">
         <v>93</v>
       </c>
@@ -3477,7 +4266,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5">
       <c r="A22" s="8" t="s">
         <v>94</v>
       </c>
@@ -3491,7 +4280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5">
       <c r="A23" s="8" t="s">
         <v>95</v>
       </c>
@@ -3505,7 +4294,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5">
       <c r="A24" s="9" t="s">
         <v>96</v>
       </c>
@@ -3519,7 +4308,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5">
       <c r="A25" s="9" t="s">
         <v>97</v>
       </c>
@@ -3533,7 +4322,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5">
       <c r="A26" s="9" t="s">
         <v>98</v>
       </c>
@@ -3547,7 +4336,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5">
       <c r="A27" s="9" t="s">
         <v>99</v>
       </c>
@@ -3561,7 +4350,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5">
       <c r="A28" s="9" t="s">
         <v>100</v>
       </c>
@@ -3575,7 +4364,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5">
       <c r="A29" s="9" t="s">
         <v>101</v>
       </c>
@@ -3589,7 +4378,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5">
       <c r="A30" s="9" t="s">
         <v>102</v>
       </c>
@@ -3603,7 +4392,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5">
       <c r="A31" s="9" t="s">
         <v>103</v>
       </c>
@@ -3617,7 +4406,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5">
       <c r="A32" s="9" t="s">
         <v>104</v>
       </c>
@@ -3631,7 +4420,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5">
       <c r="A33" s="9" t="s">
         <v>105</v>
       </c>
@@ -3645,7 +4434,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5">
       <c r="A34" s="17" t="s">
         <v>106</v>
       </c>
@@ -3659,7 +4448,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5">
       <c r="A35" s="17" t="s">
         <v>107</v>
       </c>
@@ -3673,7 +4462,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5">
       <c r="A36" s="8" t="s">
         <v>108</v>
       </c>
@@ -3687,7 +4476,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5">
       <c r="A37" s="8" t="s">
         <v>109</v>
       </c>
@@ -3701,7 +4490,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5">
       <c r="A38" s="8" t="s">
         <v>110</v>
       </c>
@@ -3715,7 +4504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5">
       <c r="A39" s="8" t="s">
         <v>111</v>
       </c>
@@ -3729,7 +4518,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5">
       <c r="A40" s="8" t="s">
         <v>112</v>
       </c>
@@ -3743,7 +4532,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5">
       <c r="A41" s="8" t="s">
         <v>113</v>
       </c>
@@ -3757,7 +4546,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5">
       <c r="A42" s="9" t="s">
         <v>114</v>
       </c>
@@ -3771,7 +4560,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5">
       <c r="A43" s="9" t="s">
         <v>115</v>
       </c>
@@ -3785,7 +4574,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5">
       <c r="A44" s="8" t="s">
         <v>116</v>
       </c>
@@ -3799,7 +4588,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5">
       <c r="A45" s="9" t="s">
         <v>117</v>
       </c>
@@ -3813,7 +4602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5">
       <c r="A46" s="9" t="s">
         <v>118</v>
       </c>
@@ -3827,7 +4616,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5">
       <c r="A47" s="16" t="s">
         <v>119</v>
       </c>
@@ -3841,7 +4630,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5">
       <c r="A48" s="16" t="s">
         <v>120</v>
       </c>
@@ -3855,7 +4644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5">
       <c r="A49" s="16" t="s">
         <v>121</v>
       </c>
@@ -3869,7 +4658,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5">
       <c r="A50" s="16" t="s">
         <v>122</v>
       </c>
@@ -3883,7 +4672,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5">
       <c r="A51" s="16" t="s">
         <v>123</v>
       </c>
@@ -3897,7 +4686,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5">
       <c r="A52" s="9" t="s">
         <v>76</v>
       </c>
@@ -3911,7 +4700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5">
       <c r="A53" s="9" t="s">
         <v>80</v>
       </c>
@@ -3925,7 +4714,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5">
       <c r="A54" s="9" t="s">
         <v>81</v>
       </c>
@@ -3939,7 +4728,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5">
       <c r="A55" s="9" t="s">
         <v>76</v>
       </c>
@@ -3953,7 +4742,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5">
       <c r="A56" s="9" t="s">
         <v>80</v>
       </c>
@@ -3967,7 +4756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5">
       <c r="A57" s="9" t="s">
         <v>81</v>
       </c>
@@ -3990,14 +4779,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F44C5BE1-96A8-884B-83A6-CAC11DBA4379}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="61.1640625" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4017,7 +4806,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
         <v>128</v>
       </c>
@@ -4031,7 +4820,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
         <v>129</v>
       </c>
@@ -4045,7 +4834,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="6" t="s">
         <v>130</v>
       </c>
@@ -4059,7 +4848,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="6" t="s">
         <v>131</v>
       </c>
@@ -4073,7 +4862,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="6" t="s">
         <v>132</v>
       </c>
@@ -4087,7 +4876,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="6" t="s">
         <v>133</v>
       </c>
@@ -4101,7 +4890,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="6" t="s">
         <v>134</v>
       </c>
@@ -4115,7 +4904,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="31">
       <c r="A9" s="6" t="s">
         <v>135</v>
       </c>
@@ -4129,7 +4918,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="6" t="s">
         <v>136</v>
       </c>
@@ -4143,7 +4932,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="31">
       <c r="A11" s="6" t="s">
         <v>137</v>
       </c>
@@ -4157,7 +4946,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
         <v>138</v>
       </c>
@@ -4171,7 +4960,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
         <v>139</v>
       </c>
@@ -4185,7 +4974,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="8" t="s">
         <v>140</v>
       </c>
@@ -4199,7 +4988,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="8" t="s">
         <v>141</v>
       </c>
@@ -4213,7 +5002,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" s="6" t="s">
         <v>142</v>
       </c>
@@ -4227,7 +5016,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="6" t="s">
         <v>143</v>
       </c>
@@ -4250,7 +5039,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{728711BE-F6C8-5D48-A4F8-3BE533FA0A66}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="77.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -4258,7 +5047,7 @@
     <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4278,7 +5067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" s="18" t="s">
         <v>144</v>
       </c>
@@ -4292,7 +5081,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" s="18" t="s">
         <v>145</v>
       </c>
@@ -4306,7 +5095,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" s="18" t="s">
         <v>146</v>
       </c>
@@ -4320,7 +5109,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" s="18" t="s">
         <v>147</v>
       </c>
@@ -4334,7 +5123,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" s="18" t="s">
         <v>148</v>
       </c>
@@ -4348,7 +5137,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" s="18" t="s">
         <v>149</v>
       </c>
@@ -4362,7 +5151,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" s="18" t="s">
         <v>150</v>
       </c>
@@ -4376,7 +5165,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" s="18" t="s">
         <v>151</v>
       </c>
@@ -4390,7 +5179,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" s="18" t="s">
         <v>152</v>
       </c>
@@ -4404,7 +5193,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" s="18" t="s">
         <v>153</v>
       </c>
@@ -4418,7 +5207,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" s="18" t="s">
         <v>154</v>
       </c>
@@ -4432,7 +5221,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" s="18" t="s">
         <v>155</v>
       </c>
@@ -4446,7 +5235,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" s="18" t="s">
         <v>156</v>
       </c>
@@ -4460,7 +5249,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" s="18" t="s">
         <v>154</v>
       </c>
@@ -4474,7 +5263,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" s="18" t="s">
         <v>155</v>
       </c>
@@ -4488,7 +5277,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5">
       <c r="A17" s="18" t="s">
         <v>156</v>
       </c>
@@ -4502,7 +5291,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5">
       <c r="A18" s="18" t="s">
         <v>157</v>
       </c>
@@ -4516,7 +5305,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5">
       <c r="A19" s="18" t="s">
         <v>158</v>
       </c>
@@ -4530,7 +5319,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5">
       <c r="A20" s="18" t="s">
         <v>159</v>
       </c>
@@ -4544,7 +5333,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5">
       <c r="A21" s="18" t="s">
         <v>160</v>
       </c>
@@ -4558,7 +5347,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5">
       <c r="A22" s="18" t="s">
         <v>161</v>
       </c>
@@ -4572,7 +5361,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5">
       <c r="A23" s="18" t="s">
         <v>162</v>
       </c>
@@ -4586,7 +5375,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5">
       <c r="A24" s="18" t="s">
         <v>163</v>
       </c>
@@ -4600,7 +5389,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5">
       <c r="A25" s="18" t="s">
         <v>164</v>
       </c>
@@ -4614,7 +5403,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5">
       <c r="A26" s="18" t="s">
         <v>165</v>
       </c>
@@ -4628,7 +5417,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5">
       <c r="A27" s="19" t="s">
         <v>166</v>
       </c>
@@ -4642,7 +5431,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5">
       <c r="A28" s="19" t="s">
         <v>167</v>
       </c>
@@ -4656,7 +5445,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5">
       <c r="A29" s="19" t="s">
         <v>168</v>
       </c>
@@ -4678,7 +5467,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B68ED0-EA25-1F47-BECA-5098C32E48E2}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="67.33203125" style="17" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -4688,7 +5477,7 @@
     <col min="7" max="7" width="25.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -4714,7 +5503,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="31">
       <c r="A2" s="21" t="s">
         <v>169</v>
       </c>
@@ -4734,7 +5523,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="31">
       <c r="A3" s="21" t="s">
         <v>170</v>
       </c>
@@ -4754,7 +5543,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="31">
       <c r="A4" s="21" t="s">
         <v>171</v>
       </c>
@@ -4774,7 +5563,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="31">
       <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
@@ -4794,7 +5583,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8">
       <c r="A6" s="21" t="s">
         <v>173</v>
       </c>
@@ -4814,7 +5603,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8">
       <c r="A7" s="21" t="s">
         <v>174</v>
       </c>
@@ -4834,7 +5623,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8">
       <c r="A8" s="21" t="s">
         <v>175</v>
       </c>
@@ -4854,7 +5643,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8">
       <c r="A9" s="21" t="s">
         <v>176</v>
       </c>
@@ -4874,7 +5663,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="31">
       <c r="A10" s="21" t="s">
         <v>177</v>
       </c>
@@ -4894,7 +5683,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="31">
       <c r="A11" s="21" t="s">
         <v>178</v>
       </c>
@@ -4914,7 +5703,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8">
       <c r="A12" s="21" t="s">
         <v>179</v>
       </c>
@@ -4934,7 +5723,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="31">
       <c r="A13" s="21" t="s">
         <v>180</v>
       </c>
@@ -4954,7 +5743,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="31">
       <c r="A14" s="21" t="s">
         <v>181</v>
       </c>
@@ -4974,7 +5763,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="31">
       <c r="A15" s="21" t="s">
         <v>182</v>
       </c>
@@ -4994,7 +5783,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="31">
       <c r="A16" s="21" t="s">
         <v>183</v>
       </c>
@@ -5014,7 +5803,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8">
       <c r="A17" s="21" t="s">
         <v>184</v>
       </c>
@@ -5034,7 +5823,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="31">
       <c r="A18" s="21" t="s">
         <v>185</v>
       </c>
@@ -5054,7 +5843,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="31">
       <c r="A19" s="21" t="s">
         <v>189</v>
       </c>
@@ -5074,7 +5863,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="31">
       <c r="A20" s="21" t="s">
         <v>190</v>
       </c>
@@ -5094,7 +5883,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="31">
       <c r="A21" s="8" t="s">
         <v>191</v>
       </c>
@@ -5114,7 +5903,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="31">
       <c r="A22" s="21" t="s">
         <v>192</v>
       </c>
@@ -5134,7 +5923,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="31">
       <c r="A23" s="8" t="s">
         <v>193</v>
       </c>
@@ -5154,7 +5943,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="31">
       <c r="A24" s="8" t="s">
         <v>194</v>
       </c>
@@ -5174,7 +5963,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8">
       <c r="A25" s="8" t="s">
         <v>195</v>
       </c>
@@ -5194,7 +5983,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" ht="31">
       <c r="A26" s="8" t="s">
         <v>196</v>
       </c>
@@ -5214,7 +6003,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" ht="31">
       <c r="A27" s="8" t="s">
         <v>197</v>
       </c>
@@ -5234,7 +6023,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" ht="31">
       <c r="A28" s="8" t="s">
         <v>198</v>
       </c>
@@ -5254,7 +6043,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="31">
       <c r="A29" s="21" t="s">
         <v>199</v>
       </c>
@@ -5274,7 +6063,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8">
       <c r="A30" s="21" t="s">
         <v>200</v>
       </c>
@@ -5294,7 +6083,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="31">
       <c r="A31" s="21" t="s">
         <v>201</v>
       </c>
@@ -5314,7 +6103,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8">
       <c r="A32" s="21" t="s">
         <v>202</v>
       </c>
@@ -5334,7 +6123,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="31">
       <c r="A33" s="21" t="s">
         <v>203</v>
       </c>
@@ -5354,7 +6143,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8">
       <c r="A34" s="8" t="s">
         <v>204</v>
       </c>
@@ -5374,7 +6163,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="31">
       <c r="A35" s="8" t="s">
         <v>205</v>
       </c>
@@ -5394,7 +6183,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8">
       <c r="A36" s="8" t="s">
         <v>206</v>
       </c>
@@ -5414,7 +6203,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8">
       <c r="A37" s="8" t="s">
         <v>207</v>
       </c>
@@ -5443,7 +6232,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC2276F-B0B8-6047-8DEC-2FD310B59F97}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -5454,7 +6243,7 @@
     <col min="8" max="8" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -5480,7 +6269,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="77.5">
       <c r="A2" s="21" t="s">
         <v>169</v>
       </c>
@@ -5500,7 +6289,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="77.5">
       <c r="A3" s="21" t="s">
         <v>170</v>
       </c>
@@ -5520,7 +6309,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="77.5">
       <c r="A4" s="21" t="s">
         <v>171</v>
       </c>
@@ -5540,7 +6329,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="108.5">
       <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
@@ -5560,7 +6349,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="46.5">
       <c r="A6" s="21" t="s">
         <v>173</v>
       </c>
@@ -5580,7 +6369,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="46.5">
       <c r="A7" s="21" t="s">
         <v>174</v>
       </c>
@@ -5600,7 +6389,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="62">
       <c r="A8" s="21" t="s">
         <v>175</v>
       </c>
@@ -5620,7 +6409,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="62">
       <c r="A9" s="21" t="s">
         <v>176</v>
       </c>
@@ -5640,7 +6429,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="108.5">
       <c r="A10" s="21" t="s">
         <v>177</v>
       </c>
@@ -5660,7 +6449,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="93">
       <c r="A11" s="21" t="s">
         <v>178</v>
       </c>
@@ -5680,7 +6469,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="77.5">
       <c r="A12" s="21" t="s">
         <v>179</v>
       </c>
@@ -5700,7 +6489,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="93">
       <c r="A13" s="21" t="s">
         <v>180</v>
       </c>
@@ -5720,7 +6509,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="77.5">
       <c r="A14" s="21" t="s">
         <v>181</v>
       </c>
@@ -5740,7 +6529,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="77.5">
       <c r="A15" s="21" t="s">
         <v>182</v>
       </c>
@@ -5760,7 +6549,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="77.5">
       <c r="A16" s="21" t="s">
         <v>183</v>
       </c>
@@ -5780,7 +6569,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" ht="62">
       <c r="A17" s="21" t="s">
         <v>184</v>
       </c>
@@ -5800,7 +6589,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="93">
       <c r="A18" s="21" t="s">
         <v>185</v>
       </c>
@@ -5820,7 +6609,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="93">
       <c r="A19" s="21" t="s">
         <v>189</v>
       </c>
@@ -5840,7 +6629,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="108.5">
       <c r="A20" s="21" t="s">
         <v>190</v>
       </c>
@@ -5860,7 +6649,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="93">
       <c r="A21" s="8" t="s">
         <v>191</v>
       </c>
@@ -5880,7 +6669,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="93">
       <c r="A22" s="21" t="s">
         <v>192</v>
       </c>
@@ -5900,7 +6689,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="108.5">
       <c r="A23" s="8" t="s">
         <v>193</v>
       </c>
@@ -5920,7 +6709,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="93">
       <c r="A24" s="8" t="s">
         <v>194</v>
       </c>
@@ -5940,7 +6729,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="62">
       <c r="A25" s="8" t="s">
         <v>195</v>
       </c>
@@ -5960,7 +6749,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" ht="77.5">
       <c r="A26" s="8" t="s">
         <v>196</v>
       </c>
@@ -5980,7 +6769,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" ht="93">
       <c r="A27" s="8" t="s">
         <v>197</v>
       </c>
@@ -6000,7 +6789,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" ht="93">
       <c r="A28" s="8" t="s">
         <v>198</v>
       </c>
@@ -6020,7 +6809,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="77.5">
       <c r="A29" s="21" t="s">
         <v>199</v>
       </c>
@@ -6040,7 +6829,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="62">
       <c r="A30" s="21" t="s">
         <v>200</v>
       </c>
@@ -6060,7 +6849,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="77.5">
       <c r="A31" s="21" t="s">
         <v>201</v>
       </c>
@@ -6080,7 +6869,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="62">
       <c r="A32" s="21" t="s">
         <v>202</v>
       </c>
@@ -6100,7 +6889,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="77.5">
       <c r="A33" s="21" t="s">
         <v>203</v>
       </c>
@@ -6120,7 +6909,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" ht="62">
       <c r="A34" s="8" t="s">
         <v>204</v>
       </c>
@@ -6140,7 +6929,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="77.5">
       <c r="A35" s="8" t="s">
         <v>205</v>
       </c>
@@ -6160,7 +6949,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" ht="46.5">
       <c r="A36" s="8" t="s">
         <v>206</v>
       </c>
@@ -6180,7 +6969,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="62">
       <c r="A37" s="8" t="s">
         <v>207</v>
       </c>
@@ -6208,14 +6997,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125867D4-4268-FD46-BD8D-BFA58B4600F1}">
   <dimension ref="A1:H37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -6241,7 +7030,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="170.5">
       <c r="A2" s="21" t="s">
         <v>169</v>
       </c>
@@ -6261,7 +7050,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ht="155">
       <c r="A3" s="21" t="s">
         <v>170</v>
       </c>
@@ -6281,7 +7070,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ht="155">
       <c r="A4" s="21" t="s">
         <v>171</v>
       </c>
@@ -6301,7 +7090,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="255" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="232.5">
       <c r="A5" s="21" t="s">
         <v>172</v>
       </c>
@@ -6321,7 +7110,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ht="77.5">
       <c r="A6" s="21" t="s">
         <v>173</v>
       </c>
@@ -6341,7 +7130,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ht="93">
       <c r="A7" s="21" t="s">
         <v>174</v>
       </c>
@@ -6361,7 +7150,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ht="124">
       <c r="A8" s="21" t="s">
         <v>175</v>
       </c>
@@ -6381,7 +7170,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="124">
       <c r="A9" s="21" t="s">
         <v>176</v>
       </c>
@@ -6401,7 +7190,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ht="186">
       <c r="A10" s="21" t="s">
         <v>177</v>
       </c>
@@ -6421,7 +7210,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="170.5">
       <c r="A11" s="21" t="s">
         <v>178</v>
       </c>
@@ -6441,7 +7230,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ht="124">
       <c r="A12" s="21" t="s">
         <v>179</v>
       </c>
@@ -6461,7 +7250,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ht="170.5">
       <c r="A13" s="21" t="s">
         <v>180</v>
       </c>
@@ -6481,7 +7270,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ht="155">
       <c r="A14" s="21" t="s">
         <v>181</v>
       </c>
@@ -6501,7 +7290,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ht="139.5">
       <c r="A15" s="21" t="s">
         <v>182</v>
       </c>
@@ -6521,7 +7310,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ht="155">
       <c r="A16" s="21" t="s">
         <v>183</v>
       </c>
@@ -6541,7 +7330,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" ht="93">
       <c r="A17" s="21" t="s">
         <v>184</v>
       </c>
@@ -6561,7 +7350,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" ht="186">
       <c r="A18" s="21" t="s">
         <v>185</v>
       </c>
@@ -6581,7 +7370,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" ht="155">
       <c r="A19" s="21" t="s">
         <v>189</v>
       </c>
@@ -6601,7 +7390,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="238" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" ht="186">
       <c r="A20" s="21" t="s">
         <v>190</v>
       </c>
@@ -6621,7 +7410,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" ht="186">
       <c r="A21" s="8" t="s">
         <v>191</v>
       </c>
@@ -6641,7 +7430,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="139.5">
       <c r="A22" s="21" t="s">
         <v>192</v>
       </c>
@@ -6661,7 +7450,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="238" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="217">
       <c r="A23" s="8" t="s">
         <v>193</v>
       </c>
@@ -6681,7 +7470,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" ht="170.5">
       <c r="A24" s="8" t="s">
         <v>194</v>
       </c>
@@ -6701,7 +7490,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" ht="124">
       <c r="A25" s="8" t="s">
         <v>195</v>
       </c>
@@ -6721,7 +7510,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" ht="155">
       <c r="A26" s="8" t="s">
         <v>196</v>
       </c>
@@ -6741,7 +7530,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" ht="139.5">
       <c r="A27" s="8" t="s">
         <v>197</v>
       </c>
@@ -6761,7 +7550,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" ht="170.5">
       <c r="A28" s="8" t="s">
         <v>198</v>
       </c>
@@ -6781,7 +7570,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="139.5">
       <c r="A29" s="21" t="s">
         <v>199</v>
       </c>
@@ -6801,7 +7590,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="124">
       <c r="A30" s="21" t="s">
         <v>200</v>
       </c>
@@ -6821,7 +7610,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="155">
       <c r="A31" s="21" t="s">
         <v>201</v>
       </c>
@@ -6841,7 +7630,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="124">
       <c r="A32" s="21" t="s">
         <v>202</v>
       </c>
@@ -6861,7 +7650,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" ht="139.5">
       <c r="A33" s="21" t="s">
         <v>203</v>
       </c>
@@ -6881,7 +7670,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" ht="124">
       <c r="A34" s="8" t="s">
         <v>204</v>
       </c>
@@ -6901,7 +7690,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="153" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" ht="139.5">
       <c r="A35" s="8" t="s">
         <v>205</v>
       </c>
@@ -6921,7 +7710,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" ht="108.5">
       <c r="A36" s="8" t="s">
         <v>206</v>
       </c>
@@ -6941,7 +7730,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="124">
       <c r="A37" s="8" t="s">
         <v>207</v>
       </c>

</xml_diff>

<commit_message>
chore: Clean up unwanted files - remove debug scripts, test data, web version, and update .gitignore
</commit_message>
<xml_diff>
--- a/asana_generator_app/resources/Template.xlsx
+++ b/asana_generator_app/resources/Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sakthimx\Desktop\ASANA_Dashboard\asana_generator_app\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109D34C8-BB9E-41E0-AB96-8FF846F700B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F2BF5B-8589-44C6-9EDC-B6F87DAF0FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="11" activeTab="15" xr2:uid="{65F45C9F-47C9-5D42-9768-363B1ABC41FB}"/>
   </bookViews>
@@ -1382,7 +1382,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" s="5">
         <v>2.0833333333333332E-2</v>
@@ -2291,7 +2291,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31">
+    <row r="2" spans="1:6">
       <c r="A2" s="25" t="s">
         <v>80</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="31">
+    <row r="3" spans="1:6">
       <c r="A3" s="25" t="s">
         <v>81</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="46.5">
+    <row r="4" spans="1:6" ht="31">
       <c r="A4" s="25" t="s">
         <v>135</v>
       </c>
@@ -2324,7 +2324,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="31">
+    <row r="5" spans="1:6">
       <c r="A5" s="25" t="s">
         <v>160</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="31">
+    <row r="6" spans="1:6">
       <c r="A6" s="25" t="s">
         <v>161</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="46.5">
+    <row r="7" spans="1:6">
       <c r="A7" s="25" t="s">
         <v>162</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="46.5">
+    <row r="8" spans="1:6">
       <c r="A8" s="25" t="s">
         <v>163</v>
       </c>
@@ -2368,7 +2368,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="46.5">
+    <row r="9" spans="1:6">
       <c r="A9" s="25" t="s">
         <v>164</v>
       </c>
@@ -2379,7 +2379,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="46.5">
+    <row r="10" spans="1:6">
       <c r="A10" s="25" t="s">
         <v>165</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="62">
+    <row r="11" spans="1:6" ht="31">
       <c r="A11" s="25" t="s">
         <v>250</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="31">
+    <row r="12" spans="1:6">
       <c r="A12" s="25" t="s">
         <v>210</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="46.5">
+    <row r="15" spans="1:6">
       <c r="A15" s="25" t="s">
         <v>251</v>
       </c>
@@ -2445,7 +2445,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="46.5">
+    <row r="16" spans="1:6">
       <c r="A16" s="25" t="s">
         <v>252</v>
       </c>
@@ -2456,7 +2456,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="46.5">
+    <row r="17" spans="1:5">
       <c r="A17" s="25" t="s">
         <v>253</v>
       </c>
@@ -2467,7 +2467,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="46.5">
+    <row r="18" spans="1:5">
       <c r="A18" s="25" t="s">
         <v>254</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="31">
+    <row r="19" spans="1:5">
       <c r="A19" s="25" t="s">
         <v>210</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="62">
+    <row r="22" spans="1:5" ht="31">
       <c r="A22" s="25" t="s">
         <v>220</v>
       </c>
@@ -2522,7 +2522,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="62">
+    <row r="23" spans="1:5" ht="31">
       <c r="A23" s="25" t="s">
         <v>221</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="62">
+    <row r="24" spans="1:5">
       <c r="A24" s="25" t="s">
         <v>222</v>
       </c>
@@ -2544,7 +2544,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="77.5">
+    <row r="25" spans="1:5" ht="31">
       <c r="A25" s="25" t="s">
         <v>223</v>
       </c>
@@ -2555,7 +2555,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="46.5">
+    <row r="26" spans="1:5">
       <c r="A26" s="25" t="s">
         <v>224</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="77.5">
+    <row r="27" spans="1:5" ht="31">
       <c r="A27" s="25" t="s">
         <v>225</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="77.5">
+    <row r="28" spans="1:5" ht="31">
       <c r="A28" s="25" t="s">
         <v>226</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="62">
+    <row r="29" spans="1:5">
       <c r="A29" s="25" t="s">
         <v>227</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="77.5">
+    <row r="30" spans="1:5" ht="31">
       <c r="A30" s="25" t="s">
         <v>228</v>
       </c>
@@ -2610,7 +2610,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="31">
+    <row r="31" spans="1:5">
       <c r="A31" s="25" t="s">
         <v>229</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="31">
+    <row r="32" spans="1:5">
       <c r="A32" s="25" t="s">
         <v>230</v>
       </c>
@@ -2632,7 +2632,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="46.5">
+    <row r="33" spans="1:5">
       <c r="A33" s="25" t="s">
         <v>231</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="46.5">
+    <row r="34" spans="1:5">
       <c r="A34" s="25" t="s">
         <v>232</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="62">
+    <row r="35" spans="1:5" ht="31">
       <c r="A35" s="25" t="s">
         <v>233</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="62">
+    <row r="36" spans="1:5" ht="31">
       <c r="A36" s="25" t="s">
         <v>234</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="77.5">
+    <row r="37" spans="1:5" ht="31">
       <c r="A37" s="25" t="s">
         <v>235</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="62">
+    <row r="38" spans="1:5" ht="31">
       <c r="A38" s="25" t="s">
         <v>236</v>
       </c>
@@ -2698,7 +2698,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="93">
+    <row r="39" spans="1:5" ht="31">
       <c r="A39" s="25" t="s">
         <v>237</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="93">
+    <row r="40" spans="1:5" ht="31">
       <c r="A40" s="25" t="s">
         <v>178</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="77.5">
+    <row r="41" spans="1:5" ht="31">
       <c r="A41" s="25" t="s">
         <v>255</v>
       </c>
@@ -2731,7 +2731,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="93">
+    <row r="42" spans="1:5" ht="31">
       <c r="A42" s="25" t="s">
         <v>198</v>
       </c>
@@ -2742,7 +2742,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="62">
+    <row r="43" spans="1:5" ht="31">
       <c r="A43" s="25" t="s">
         <v>256</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="77.5">
+    <row r="44" spans="1:5" ht="31">
       <c r="A44" s="25" t="s">
         <v>200</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="93">
+    <row r="45" spans="1:5" ht="31">
       <c r="A45" s="25" t="s">
         <v>257</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="93">
+    <row r="46" spans="1:5" ht="31">
       <c r="A46" s="25" t="s">
         <v>258</v>
       </c>
@@ -2786,7 +2786,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="77.5">
+    <row r="47" spans="1:5" ht="31">
       <c r="A47" s="25" t="s">
         <v>259</v>
       </c>
@@ -2797,7 +2797,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="77.5">
+    <row r="48" spans="1:5" ht="31">
       <c r="A48" s="25" t="s">
         <v>260</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="77.5">
+    <row r="49" spans="1:5" ht="31">
       <c r="A49" s="25" t="s">
         <v>261</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="62">
+    <row r="50" spans="1:5" ht="31">
       <c r="A50" s="25" t="s">
         <v>184</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="93">
+    <row r="51" spans="1:5" ht="31">
       <c r="A51" s="25" t="s">
         <v>185</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="93">
+    <row r="52" spans="1:5" ht="31">
       <c r="A52" s="25" t="s">
         <v>189</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="108.5">
+    <row r="53" spans="1:5" ht="46.5">
       <c r="A53" s="25" t="s">
         <v>190</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="108.5">
+    <row r="54" spans="1:5" ht="31">
       <c r="A54" s="25" t="s">
         <v>262</v>
       </c>
@@ -2874,7 +2874,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="93">
+    <row r="55" spans="1:5" ht="31">
       <c r="A55" s="25" t="s">
         <v>263</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="108.5">
+    <row r="56" spans="1:5" ht="46.5">
       <c r="A56" s="25" t="s">
         <v>193</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="93">
+    <row r="57" spans="1:5" ht="31">
       <c r="A57" s="25" t="s">
         <v>194</v>
       </c>
@@ -2907,7 +2907,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="62">
+    <row r="58" spans="1:5" ht="31">
       <c r="A58" s="25" t="s">
         <v>195</v>
       </c>
@@ -2918,7 +2918,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="77.5">
+    <row r="59" spans="1:5" ht="31">
       <c r="A59" s="25" t="s">
         <v>196</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="62">
+    <row r="60" spans="1:5" ht="31">
       <c r="A60" s="25" t="s">
         <v>202</v>
       </c>
@@ -2940,7 +2940,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="77.5">
+    <row r="61" spans="1:5" ht="31">
       <c r="A61" s="25" t="s">
         <v>203</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="62">
+    <row r="62" spans="1:5" ht="31">
       <c r="A62" s="25" t="s">
         <v>204</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="77.5">
+    <row r="63" spans="1:5" ht="31">
       <c r="A63" s="25" t="s">
         <v>205</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="62">
+    <row r="64" spans="1:5">
       <c r="A64" s="25" t="s">
         <v>206</v>
       </c>
@@ -2984,7 +2984,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="62">
+    <row r="65" spans="1:5" ht="31">
       <c r="A65" s="25" t="s">
         <v>207</v>
       </c>

</xml_diff>

<commit_message>
feat: config-driven architecture, settings tab, assignee feature, dialog button fix
- Added config.json as single source of truth for devices, CSV fields, display columns, export headers, thresholds, and assignees
- Created ConfigManager singleton (core/config_manager.py) with typed accessors
- Added Settings tab (ui/settings_dialog.py) with 6 sub-tabs: Devices, CSV Fields, Display Columns, Export Headers, Thresholds, Assignees
- Refactored main_window.py: DEVICES and export HEADERS now config-driven
- Refactored csv_importer.py: KEY_COLUMNS, iteration fields, thresholds from config
- Refactored report_generator_tab.py: display columns from config
- Added Assignee dropdown in Task Creator (shows name, exports email to Assignee Email column)
- Fixed dialog button visibility: Fusion style + QSS dark text defaults
- All changes persist to config.json - zero code changes needed for future devices/fields
</commit_message>
<xml_diff>
--- a/asana_generator_app/resources/Template.xlsx
+++ b/asana_generator_app/resources/Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sakthimx\Desktop\ASANA_Dashboard\asana_generator_app\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sakthimx\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F2BF5B-8589-44C6-9EDC-B6F87DAF0FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9EE6E2-28EA-4D22-9D1D-186DCDDF348F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="11" activeTab="15" xr2:uid="{65F45C9F-47C9-5D42-9768-363B1ABC41FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{65F45C9F-47C9-5D42-9768-363B1ABC41FB}"/>
   </bookViews>
   <sheets>
     <sheet name="P0" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="274">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -587,9 +587,6 @@
     <t>Decanter OOBE - Time taken to load 'Registration' screen when 'Next' button is clicked in WiFi set-up screen.</t>
   </si>
   <si>
-    <t>Decanter OOBE - Time taken to load 'Welcome' screen from Registration screen.</t>
-  </si>
-  <si>
     <t>Decanter OOBE - Time taken to load 'Goodreads sign-in / Sign-up' page from 'Get the Kindle App' screen</t>
   </si>
   <si>
@@ -641,15 +638,9 @@
     <t>Decanter OOBE - Time taken to load Prime upsell page from Audible 'Upsell' page</t>
   </si>
   <si>
-    <t>Decanter OOBE - Time taken to load 'Two Step Verification' page from registration page</t>
-  </si>
-  <si>
     <t>Decanter OOBE - Time taken to load 'Send verification code' page from 'Two Step Verification' page</t>
   </si>
   <si>
-    <t>Decanter OOBE - Time taken to load 'Verify Account' page from registration page.</t>
-  </si>
-  <si>
     <t>Decanter OOBE - Time taken to display code when 'Create code' is clicked.</t>
   </si>
   <si>
@@ -843,6 +834,42 @@
   </si>
   <si>
     <t>Rossini,Seabreeze,Calvados,Pisco</t>
+  </si>
+  <si>
+    <t>From setting tap exisiting account going to registration screen</t>
+  </si>
+  <si>
+    <t>From setting - Time taken to load 'Password' screen from Registration screen.</t>
+  </si>
+  <si>
+    <t>From setting - Time taken to complete registration and land on load 'setting page' from password screen.</t>
+  </si>
+  <si>
+    <t>From setting - Time taken to load 'Two Step Verification' page from password page</t>
+  </si>
+  <si>
+    <t>From Setting - Time taken to load 'Verify Account' page from password page.</t>
+  </si>
+  <si>
+    <t>From setting - Time taken to display code when 'Create code' is clicked.</t>
+  </si>
+  <si>
+    <t>Time taken for change region popup appears in" verify account page"</t>
+  </si>
+  <si>
+    <t>Time taken for change region to reflect in "verify account page"</t>
+  </si>
+  <si>
+    <t>From setting - Time taken to load 'Verify Account' page from Registration page.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Password' screen from Registration screen.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE - Time taken to load 'Welcome' screen from password screen.</t>
+  </si>
+  <si>
+    <t>Decanter OOBE Time taken to load 'Verify Account' page from Registration page.</t>
   </si>
 </sst>
 </file>
@@ -1482,10 +1509,10 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E2" s="12">
         <v>15</v>
@@ -1496,10 +1523,10 @@
         <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E3" s="12">
         <v>15</v>
@@ -1510,10 +1537,10 @@
         <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E4" s="12">
         <v>10</v>
@@ -1521,13 +1548,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="24" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D5" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E5" s="12">
         <v>10</v>
@@ -1535,13 +1562,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="24" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D6" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E6" s="12">
         <v>10</v>
@@ -1552,10 +1579,10 @@
         <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E7" s="12">
         <v>15</v>
@@ -1566,10 +1593,10 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D8" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E8" s="12">
         <v>15</v>
@@ -1580,10 +1607,10 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D9" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E9" s="12">
         <v>10</v>
@@ -1591,13 +1618,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C10" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E10" s="12">
         <v>10</v>
@@ -1605,13 +1632,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C11" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D11" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E11" s="12">
         <v>10</v>
@@ -1654,13 +1681,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="9" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E2" s="12">
         <v>22</v>
@@ -1668,13 +1695,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C3" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E3" s="12">
         <v>22</v>
@@ -1682,13 +1709,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C4" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E4" s="12">
         <v>22</v>
@@ -1696,13 +1723,13 @@
     </row>
     <row r="5" spans="1:6" ht="31">
       <c r="A5" s="9" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C5" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E5" s="12">
         <v>22</v>
@@ -1710,13 +1737,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C6" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E6" s="12">
         <v>22</v>
@@ -1724,13 +1751,13 @@
     </row>
     <row r="7" spans="1:6" ht="31">
       <c r="A7" s="9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C7" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E7" s="12">
         <v>22</v>
@@ -1738,13 +1765,13 @@
     </row>
     <row r="8" spans="1:6" ht="31">
       <c r="A8" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C8" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E8" s="12">
         <v>22</v>
@@ -1752,13 +1779,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C9" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E9" s="12">
         <v>22</v>
@@ -1766,13 +1793,13 @@
     </row>
     <row r="10" spans="1:6" ht="31">
       <c r="A10" s="9" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C10" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E10" s="12">
         <v>22</v>
@@ -1780,13 +1807,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C11" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E11" s="12">
         <v>22</v>
@@ -1794,13 +1821,13 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C12" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E12" s="12">
         <v>22</v>
@@ -1808,13 +1835,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C13" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D13" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E13" s="12">
         <v>22</v>
@@ -1822,13 +1849,13 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="9" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C14" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D14" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E14" s="12">
         <v>22</v>
@@ -1836,13 +1863,13 @@
     </row>
     <row r="15" spans="1:6" ht="31">
       <c r="A15" s="9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C15" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D15" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E15" s="12">
         <v>22</v>
@@ -1850,13 +1877,13 @@
     </row>
     <row r="16" spans="1:6" ht="31">
       <c r="A16" s="9" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C16" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D16" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E16" s="12">
         <v>22</v>
@@ -1864,13 +1891,13 @@
     </row>
     <row r="17" spans="1:5" ht="31">
       <c r="A17" s="9" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C17" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D17" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E17" s="12">
         <v>22</v>
@@ -1878,13 +1905,13 @@
     </row>
     <row r="18" spans="1:5" ht="31">
       <c r="A18" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C18" t="s">
+        <v>237</v>
+      </c>
+      <c r="D18" t="s">
         <v>236</v>
-      </c>
-      <c r="C18" t="s">
-        <v>240</v>
-      </c>
-      <c r="D18" t="s">
-        <v>239</v>
       </c>
       <c r="E18" s="12">
         <v>22</v>
@@ -1892,13 +1919,13 @@
     </row>
     <row r="19" spans="1:5" ht="31">
       <c r="A19" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="C19" t="s">
         <v>237</v>
       </c>
-      <c r="C19" t="s">
-        <v>240</v>
-      </c>
       <c r="D19" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E19" s="12">
         <v>22</v>
@@ -1942,13 +1969,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="8" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C2" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E2" s="12">
         <v>40</v>
@@ -1956,13 +1983,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="8" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E3" s="12">
         <v>40</v>
@@ -1970,13 +1997,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E4" s="12">
         <v>40</v>
@@ -1984,13 +2011,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="8" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C5" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E5" s="12">
         <v>40</v>
@@ -1998,13 +2025,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E6" s="12">
         <v>40</v>
@@ -2012,13 +2039,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E7" s="12">
         <v>40</v>
@@ -2026,13 +2053,13 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C8" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E8" s="12">
         <v>40</v>
@@ -2040,13 +2067,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="8" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E9" s="12">
         <v>40</v>
@@ -2054,13 +2081,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="8" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C10" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E10" s="12">
         <v>40</v>
@@ -2068,13 +2095,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="8" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C11" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E11" s="12">
         <v>40</v>
@@ -2117,13 +2144,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="9" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E2" s="12">
         <v>15</v>
@@ -2131,13 +2158,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C3" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E3" s="12">
         <v>15</v>
@@ -2145,13 +2172,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E4" s="12">
         <v>15</v>
@@ -2159,13 +2186,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" t="s">
         <v>244</v>
       </c>
-      <c r="C5" t="s">
-        <v>247</v>
-      </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E5" s="12">
         <v>30</v>
@@ -2173,13 +2200,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C6" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D6" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E6" s="12">
         <v>30</v>
@@ -2187,13 +2214,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D7" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E7" s="12">
         <v>15</v>
@@ -2201,13 +2228,13 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C8" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E8" s="12">
         <v>15</v>
@@ -2215,13 +2242,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C9" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D9" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E9" s="12">
         <v>15</v>
@@ -2229,13 +2256,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="C10" t="s">
         <v>244</v>
       </c>
-      <c r="C10" t="s">
-        <v>247</v>
-      </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E10" s="12">
         <v>30</v>
@@ -2243,13 +2270,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C11" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E11" s="12">
         <v>30</v>
@@ -2296,7 +2323,7 @@
         <v>80</v>
       </c>
       <c r="D2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E2" s="25">
         <v>10</v>
@@ -2307,7 +2334,7 @@
         <v>81</v>
       </c>
       <c r="D3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E3" s="25">
         <v>15</v>
@@ -2318,7 +2345,7 @@
         <v>135</v>
       </c>
       <c r="D4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E4" s="25">
         <v>25</v>
@@ -2329,7 +2356,7 @@
         <v>160</v>
       </c>
       <c r="D5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E5" s="25">
         <v>30</v>
@@ -2340,7 +2367,7 @@
         <v>161</v>
       </c>
       <c r="D6" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E6" s="25">
         <v>30</v>
@@ -2351,7 +2378,7 @@
         <v>162</v>
       </c>
       <c r="D7" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E7" s="25">
         <v>30</v>
@@ -2362,7 +2389,7 @@
         <v>163</v>
       </c>
       <c r="D8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E8" s="25">
         <v>30</v>
@@ -2373,7 +2400,7 @@
         <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E9" s="25">
         <v>30</v>
@@ -2384,7 +2411,7 @@
         <v>165</v>
       </c>
       <c r="D10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E10" s="25">
         <v>30</v>
@@ -2392,10 +2419,10 @@
     </row>
     <row r="11" spans="1:6" ht="31">
       <c r="A11" s="25" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E11" s="25">
         <v>15</v>
@@ -2403,10 +2430,10 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="25" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D12" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E12" s="25">
         <v>40</v>
@@ -2414,10 +2441,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="25" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E13" s="25">
         <v>40</v>
@@ -2425,10 +2452,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="25" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D14" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E14" s="25">
         <v>40</v>
@@ -2436,10 +2463,10 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="25" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D15" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E15" s="25">
         <v>40</v>
@@ -2447,10 +2474,10 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="25" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D16" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E16" s="25">
         <v>40</v>
@@ -2458,10 +2485,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="25" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D17" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E17" s="25">
         <v>40</v>
@@ -2469,10 +2496,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="25" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D18" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E18" s="25">
         <v>40</v>
@@ -2480,10 +2507,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="25" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D19" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E19" s="25">
         <v>40</v>
@@ -2491,10 +2518,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="25" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D20" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E20" s="25">
         <v>40</v>
@@ -2502,10 +2529,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="25" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D21" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E21" s="25">
         <v>40</v>
@@ -2513,10 +2540,10 @@
     </row>
     <row r="22" spans="1:5" ht="31">
       <c r="A22" s="25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D22" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E22" s="25">
         <v>22</v>
@@ -2524,10 +2551,10 @@
     </row>
     <row r="23" spans="1:5" ht="31">
       <c r="A23" s="25" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D23" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E23" s="25">
         <v>22</v>
@@ -2535,10 +2562,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="25" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D24" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E24" s="25">
         <v>22</v>
@@ -2546,10 +2573,10 @@
     </row>
     <row r="25" spans="1:5" ht="31">
       <c r="A25" s="25" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D25" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E25" s="25">
         <v>22</v>
@@ -2557,10 +2584,10 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="25" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D26" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E26" s="25">
         <v>22</v>
@@ -2568,10 +2595,10 @@
     </row>
     <row r="27" spans="1:5" ht="31">
       <c r="A27" s="25" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D27" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E27" s="25">
         <v>22</v>
@@ -2579,10 +2606,10 @@
     </row>
     <row r="28" spans="1:5" ht="31">
       <c r="A28" s="25" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D28" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E28" s="25">
         <v>22</v>
@@ -2590,10 +2617,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="25" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D29" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E29" s="25">
         <v>22</v>
@@ -2601,10 +2628,10 @@
     </row>
     <row r="30" spans="1:5" ht="31">
       <c r="A30" s="25" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D30" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E30" s="25">
         <v>22</v>
@@ -2612,10 +2639,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="25" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D31" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E31" s="25">
         <v>22</v>
@@ -2623,10 +2650,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="25" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D32" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E32" s="25">
         <v>22</v>
@@ -2634,10 +2661,10 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="25" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D33" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E33" s="25">
         <v>22</v>
@@ -2645,10 +2672,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="25" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D34" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E34" s="25">
         <v>22</v>
@@ -2656,10 +2683,10 @@
     </row>
     <row r="35" spans="1:5" ht="31">
       <c r="A35" s="25" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D35" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E35" s="25">
         <v>22</v>
@@ -2667,10 +2694,10 @@
     </row>
     <row r="36" spans="1:5" ht="31">
       <c r="A36" s="25" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D36" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E36" s="25">
         <v>22</v>
@@ -2678,10 +2705,10 @@
     </row>
     <row r="37" spans="1:5" ht="31">
       <c r="A37" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="D37" t="s">
         <v>235</v>
-      </c>
-      <c r="D37" t="s">
-        <v>238</v>
       </c>
       <c r="E37" s="25">
         <v>22</v>
@@ -2689,10 +2716,10 @@
     </row>
     <row r="38" spans="1:5" ht="31">
       <c r="A38" s="25" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D38" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E38" s="25">
         <v>22</v>
@@ -2700,10 +2727,10 @@
     </row>
     <row r="39" spans="1:5" ht="31">
       <c r="A39" s="25" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D39" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E39" s="25">
         <v>22</v>
@@ -2714,7 +2741,7 @@
         <v>178</v>
       </c>
       <c r="D40" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E40" s="25">
         <v>30</v>
@@ -2722,10 +2749,10 @@
     </row>
     <row r="41" spans="1:5" ht="31">
       <c r="A41" s="25" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D41" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E41" s="25">
         <v>40</v>
@@ -2733,10 +2760,10 @@
     </row>
     <row r="42" spans="1:5" ht="31">
       <c r="A42" s="25" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D42" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E42" s="25">
         <v>40</v>
@@ -2744,10 +2771,10 @@
     </row>
     <row r="43" spans="1:5" ht="31">
       <c r="A43" s="25" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D43" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E43" s="25">
         <v>40</v>
@@ -2755,10 +2782,10 @@
     </row>
     <row r="44" spans="1:5" ht="31">
       <c r="A44" s="25" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D44" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E44" s="25">
         <v>40</v>
@@ -2766,10 +2793,10 @@
     </row>
     <row r="45" spans="1:5" ht="31">
       <c r="A45" s="25" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D45" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E45" s="25">
         <v>30</v>
@@ -2777,10 +2804,10 @@
     </row>
     <row r="46" spans="1:5" ht="31">
       <c r="A46" s="25" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D46" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E46" s="25">
         <v>30</v>
@@ -2788,10 +2815,10 @@
     </row>
     <row r="47" spans="1:5" ht="31">
       <c r="A47" s="25" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D47" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E47" s="25">
         <v>50</v>
@@ -2799,10 +2826,10 @@
     </row>
     <row r="48" spans="1:5" ht="31">
       <c r="A48" s="25" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D48" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E48" s="25">
         <v>50</v>
@@ -2810,10 +2837,10 @@
     </row>
     <row r="49" spans="1:5" ht="31">
       <c r="A49" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="D49" t="s">
         <v>261</v>
-      </c>
-      <c r="D49" t="s">
-        <v>264</v>
       </c>
       <c r="E49" s="25">
         <v>50</v>
@@ -2821,10 +2848,10 @@
     </row>
     <row r="50" spans="1:5" ht="31">
       <c r="A50" s="25" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D50" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E50" s="25">
         <v>0</v>
@@ -2832,10 +2859,10 @@
     </row>
     <row r="51" spans="1:5" ht="31">
       <c r="A51" s="25" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D51" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E51" s="25">
         <v>0</v>
@@ -2843,10 +2870,10 @@
     </row>
     <row r="52" spans="1:5" ht="31">
       <c r="A52" s="25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D52" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E52" s="25">
         <v>50</v>
@@ -2854,10 +2881,10 @@
     </row>
     <row r="53" spans="1:5" ht="46.5">
       <c r="A53" s="25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D53" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E53" s="25">
         <v>50</v>
@@ -2865,10 +2892,10 @@
     </row>
     <row r="54" spans="1:5" ht="31">
       <c r="A54" s="25" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D54" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E54" s="25">
         <v>30</v>
@@ -2876,10 +2903,10 @@
     </row>
     <row r="55" spans="1:5" ht="31">
       <c r="A55" s="25" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D55" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E55" s="25">
         <v>30</v>
@@ -2887,10 +2914,10 @@
     </row>
     <row r="56" spans="1:5" ht="46.5">
       <c r="A56" s="25" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D56" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E56" s="25">
         <v>60</v>
@@ -2898,10 +2925,10 @@
     </row>
     <row r="57" spans="1:5" ht="31">
       <c r="A57" s="25" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D57" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E57" s="25">
         <v>60</v>
@@ -2909,10 +2936,10 @@
     </row>
     <row r="58" spans="1:5" ht="31">
       <c r="A58" s="25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D58" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E58" s="25">
         <v>50</v>
@@ -2920,10 +2947,10 @@
     </row>
     <row r="59" spans="1:5" ht="31">
       <c r="A59" s="25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D59" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E59" s="25">
         <v>50</v>
@@ -2931,10 +2958,10 @@
     </row>
     <row r="60" spans="1:5" ht="31">
       <c r="A60" s="25" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D60" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E60" s="25">
         <v>30</v>
@@ -2942,10 +2969,10 @@
     </row>
     <row r="61" spans="1:5" ht="31">
       <c r="A61" s="25" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D61" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E61" s="25">
         <v>30</v>
@@ -2953,10 +2980,10 @@
     </row>
     <row r="62" spans="1:5" ht="31">
       <c r="A62" s="25" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D62" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E62" s="25">
         <v>30</v>
@@ -2964,10 +2991,10 @@
     </row>
     <row r="63" spans="1:5" ht="31">
       <c r="A63" s="25" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D63" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E63" s="25">
         <v>30</v>
@@ -2975,10 +3002,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="25" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D64" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E64" s="25">
         <v>30</v>
@@ -2986,10 +3013,10 @@
     </row>
     <row r="65" spans="1:5" ht="31">
       <c r="A65" s="25" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D65" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E65" s="25">
         <v>30</v>
@@ -3150,7 +3177,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8414CF9-37A4-564E-A42E-4E0D99ADC213}">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="87.1640625" bestFit="1" customWidth="1"/>
@@ -3947,6 +3974,384 @@
       </c>
       <c r="E56" s="12">
         <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>262</v>
+      </c>
+      <c r="C57" t="s">
+        <v>61</v>
+      </c>
+      <c r="D57" t="s">
+        <v>126</v>
+      </c>
+      <c r="E57" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>263</v>
+      </c>
+      <c r="C58" t="s">
+        <v>61</v>
+      </c>
+      <c r="D58" t="s">
+        <v>126</v>
+      </c>
+      <c r="E58" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>264</v>
+      </c>
+      <c r="C59" t="s">
+        <v>61</v>
+      </c>
+      <c r="D59" t="s">
+        <v>126</v>
+      </c>
+      <c r="E59" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>265</v>
+      </c>
+      <c r="C60" t="s">
+        <v>61</v>
+      </c>
+      <c r="D60" t="s">
+        <v>126</v>
+      </c>
+      <c r="E60" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>266</v>
+      </c>
+      <c r="C61" t="s">
+        <v>61</v>
+      </c>
+      <c r="D61" t="s">
+        <v>126</v>
+      </c>
+      <c r="E61" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>267</v>
+      </c>
+      <c r="C62" t="s">
+        <v>61</v>
+      </c>
+      <c r="D62" t="s">
+        <v>126</v>
+      </c>
+      <c r="E62" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>268</v>
+      </c>
+      <c r="C63" t="s">
+        <v>61</v>
+      </c>
+      <c r="D63" t="s">
+        <v>126</v>
+      </c>
+      <c r="E63" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>269</v>
+      </c>
+      <c r="C64" t="s">
+        <v>61</v>
+      </c>
+      <c r="D64" t="s">
+        <v>126</v>
+      </c>
+      <c r="E64" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" t="s">
+        <v>270</v>
+      </c>
+      <c r="C65" t="s">
+        <v>61</v>
+      </c>
+      <c r="D65" t="s">
+        <v>126</v>
+      </c>
+      <c r="E65" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" t="s">
+        <v>262</v>
+      </c>
+      <c r="C66" t="s">
+        <v>61</v>
+      </c>
+      <c r="D66" t="s">
+        <v>63</v>
+      </c>
+      <c r="E66" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
+        <v>263</v>
+      </c>
+      <c r="C67" t="s">
+        <v>61</v>
+      </c>
+      <c r="D67" t="s">
+        <v>63</v>
+      </c>
+      <c r="E67" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" t="s">
+        <v>264</v>
+      </c>
+      <c r="C68" t="s">
+        <v>61</v>
+      </c>
+      <c r="D68" t="s">
+        <v>63</v>
+      </c>
+      <c r="E68" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" t="s">
+        <v>265</v>
+      </c>
+      <c r="C69" t="s">
+        <v>61</v>
+      </c>
+      <c r="D69" t="s">
+        <v>63</v>
+      </c>
+      <c r="E69" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" t="s">
+        <v>266</v>
+      </c>
+      <c r="C70" t="s">
+        <v>61</v>
+      </c>
+      <c r="D70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E70" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" t="s">
+        <v>267</v>
+      </c>
+      <c r="C71" t="s">
+        <v>61</v>
+      </c>
+      <c r="D71" t="s">
+        <v>63</v>
+      </c>
+      <c r="E71" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" t="s">
+        <v>268</v>
+      </c>
+      <c r="C72" t="s">
+        <v>61</v>
+      </c>
+      <c r="D72" t="s">
+        <v>63</v>
+      </c>
+      <c r="E72" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" t="s">
+        <v>269</v>
+      </c>
+      <c r="C73" t="s">
+        <v>61</v>
+      </c>
+      <c r="D73" t="s">
+        <v>63</v>
+      </c>
+      <c r="E73" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" t="s">
+        <v>270</v>
+      </c>
+      <c r="C74" t="s">
+        <v>61</v>
+      </c>
+      <c r="D74" t="s">
+        <v>63</v>
+      </c>
+      <c r="E74" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" t="s">
+        <v>262</v>
+      </c>
+      <c r="C75" t="s">
+        <v>61</v>
+      </c>
+      <c r="D75" t="s">
+        <v>126</v>
+      </c>
+      <c r="E75" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" t="s">
+        <v>263</v>
+      </c>
+      <c r="C76" t="s">
+        <v>61</v>
+      </c>
+      <c r="D76" t="s">
+        <v>126</v>
+      </c>
+      <c r="E76" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" t="s">
+        <v>264</v>
+      </c>
+      <c r="C77" t="s">
+        <v>61</v>
+      </c>
+      <c r="D77" t="s">
+        <v>126</v>
+      </c>
+      <c r="E77" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" t="s">
+        <v>265</v>
+      </c>
+      <c r="C78" t="s">
+        <v>61</v>
+      </c>
+      <c r="D78" t="s">
+        <v>126</v>
+      </c>
+      <c r="E78" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" t="s">
+        <v>266</v>
+      </c>
+      <c r="C79" t="s">
+        <v>61</v>
+      </c>
+      <c r="D79" t="s">
+        <v>126</v>
+      </c>
+      <c r="E79" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" t="s">
+        <v>267</v>
+      </c>
+      <c r="C80" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80" t="s">
+        <v>126</v>
+      </c>
+      <c r="E80" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" t="s">
+        <v>268</v>
+      </c>
+      <c r="C81" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81" t="s">
+        <v>126</v>
+      </c>
+      <c r="E81" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" t="s">
+        <v>269</v>
+      </c>
+      <c r="C82" t="s">
+        <v>61</v>
+      </c>
+      <c r="D82" t="s">
+        <v>126</v>
+      </c>
+      <c r="E82" s="12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" t="s">
+        <v>270</v>
+      </c>
+      <c r="C83" t="s">
+        <v>61</v>
+      </c>
+      <c r="D83" t="s">
+        <v>126</v>
+      </c>
+      <c r="E83" s="12">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -5466,7 +5871,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B68ED0-EA25-1F47-BECA-5098C32E48E2}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="67.33203125" style="17" customWidth="1"/>
@@ -5497,10 +5902,10 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H1" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="31">
@@ -5508,7 +5913,7 @@
         <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D2" t="s">
         <v>126</v>
@@ -5517,7 +5922,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H2" t="s">
         <v>61</v>
@@ -5528,7 +5933,7 @@
         <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D3" t="s">
         <v>126</v>
@@ -5537,7 +5942,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H3" t="s">
         <v>61</v>
@@ -5548,7 +5953,7 @@
         <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D4" t="s">
         <v>126</v>
@@ -5557,7 +5962,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H4" t="s">
         <v>61</v>
@@ -5568,7 +5973,7 @@
         <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D5" t="s">
         <v>126</v>
@@ -5577,7 +5982,7 @@
         <v>30</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
@@ -5588,7 +5993,7 @@
         <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D6" t="s">
         <v>126</v>
@@ -5597,7 +6002,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H6" t="s">
         <v>61</v>
@@ -5608,7 +6013,7 @@
         <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D7" t="s">
         <v>126</v>
@@ -5617,7 +6022,7 @@
         <v>60</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H7" t="s">
         <v>61</v>
@@ -5628,7 +6033,7 @@
         <v>175</v>
       </c>
       <c r="C8" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D8" t="s">
         <v>126</v>
@@ -5637,7 +6042,7 @@
         <v>30</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H8" t="s">
         <v>61</v>
@@ -5648,7 +6053,7 @@
         <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D9" t="s">
         <v>126</v>
@@ -5657,7 +6062,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H9" t="s">
         <v>61</v>
@@ -5668,7 +6073,7 @@
         <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D10" t="s">
         <v>126</v>
@@ -5677,7 +6082,7 @@
         <v>30</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H10" t="s">
         <v>61</v>
@@ -5688,7 +6093,7 @@
         <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D11" t="s">
         <v>126</v>
@@ -5697,7 +6102,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H11" t="s">
         <v>61</v>
@@ -5705,10 +6110,10 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="21" t="s">
-        <v>179</v>
+        <v>271</v>
       </c>
       <c r="C12" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D12" t="s">
         <v>126</v>
@@ -5717,18 +6122,18 @@
         <v>30</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="31">
+    <row r="13" spans="1:8">
       <c r="A13" s="21" t="s">
-        <v>180</v>
+        <v>272</v>
       </c>
       <c r="C13" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D13" t="s">
         <v>126</v>
@@ -5737,7 +6142,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H13" t="s">
         <v>61</v>
@@ -5745,10 +6150,10 @@
     </row>
     <row r="14" spans="1:8" ht="31">
       <c r="A14" s="21" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C14" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D14" t="s">
         <v>126</v>
@@ -5757,7 +6162,7 @@
         <v>50</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H14" t="s">
         <v>61</v>
@@ -5765,10 +6170,10 @@
     </row>
     <row r="15" spans="1:8" ht="31">
       <c r="A15" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C15" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D15" t="s">
         <v>126</v>
@@ -5777,7 +6182,7 @@
         <v>50</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H15" t="s">
         <v>61</v>
@@ -5785,10 +6190,10 @@
     </row>
     <row r="16" spans="1:8" ht="31">
       <c r="A16" s="21" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D16" t="s">
         <v>126</v>
@@ -5797,18 +6202,18 @@
         <v>50</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" ht="31">
       <c r="A17" s="21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D17" t="s">
         <v>126</v>
@@ -5817,18 +6222,18 @@
         <v>0</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H17" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="31">
+    <row r="18" spans="1:8">
       <c r="A18" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C18" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D18" t="s">
         <v>126</v>
@@ -5837,7 +6242,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H18" t="s">
         <v>61</v>
@@ -5845,10 +6250,10 @@
     </row>
     <row r="19" spans="1:8" ht="31">
       <c r="A19" s="21" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C19" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D19" t="s">
         <v>126</v>
@@ -5857,18 +6262,18 @@
         <v>50</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="31">
       <c r="A20" s="21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C20" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D20" t="s">
         <v>126</v>
@@ -5877,7 +6282,7 @@
         <v>50</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
@@ -5885,10 +6290,10 @@
     </row>
     <row r="21" spans="1:8" ht="31">
       <c r="A21" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C21" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D21" t="s">
         <v>126</v>
@@ -5897,7 +6302,7 @@
         <v>30</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H21" t="s">
         <v>124</v>
@@ -5905,10 +6310,10 @@
     </row>
     <row r="22" spans="1:8" ht="31">
       <c r="A22" s="21" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C22" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D22" t="s">
         <v>126</v>
@@ -5917,7 +6322,7 @@
         <v>30</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H22" t="s">
         <v>124</v>
@@ -5925,10 +6330,10 @@
     </row>
     <row r="23" spans="1:8" ht="31">
       <c r="A23" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C23" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D23" t="s">
         <v>126</v>
@@ -5937,7 +6342,7 @@
         <v>60</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H23" t="s">
         <v>124</v>
@@ -5945,10 +6350,10 @@
     </row>
     <row r="24" spans="1:8" ht="31">
       <c r="A24" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C24" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -5957,18 +6362,18 @@
         <v>60</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" ht="31">
       <c r="A25" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C25" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D25" t="s">
         <v>126</v>
@@ -5977,18 +6382,18 @@
         <v>50</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H25" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="31">
+    <row r="26" spans="1:8">
       <c r="A26" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C26" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D26" t="s">
         <v>126</v>
@@ -5997,7 +6402,7 @@
         <v>50</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H26" t="s">
         <v>124</v>
@@ -6005,10 +6410,10 @@
     </row>
     <row r="27" spans="1:8" ht="31">
       <c r="A27" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D27" t="s">
         <v>126</v>
@@ -6017,18 +6422,18 @@
         <v>40</v>
       </c>
       <c r="G27" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="31">
       <c r="A28" s="8" t="s">
-        <v>198</v>
+        <v>252</v>
       </c>
       <c r="C28" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D28" t="s">
         <v>126</v>
@@ -6037,7 +6442,7 @@
         <v>40</v>
       </c>
       <c r="G28" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H28" t="s">
         <v>125</v>
@@ -6045,10 +6450,10 @@
     </row>
     <row r="29" spans="1:8" ht="31">
       <c r="A29" s="21" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D29" t="s">
         <v>126</v>
@@ -6057,7 +6462,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H29" t="s">
         <v>125</v>
@@ -6065,10 +6470,10 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="21" t="s">
-        <v>200</v>
+        <v>253</v>
       </c>
       <c r="C30" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D30" t="s">
         <v>126</v>
@@ -6077,18 +6482,18 @@
         <v>40</v>
       </c>
       <c r="G30" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H30" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="31">
+    <row r="31" spans="1:8">
       <c r="A31" s="21" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C31" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D31" t="s">
         <v>126</v>
@@ -6097,7 +6502,7 @@
         <v>30</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H31" t="s">
         <v>125</v>
@@ -6105,10 +6510,10 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="21" t="s">
-        <v>202</v>
+        <v>268</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D32" t="s">
         <v>126</v>
@@ -6117,18 +6522,18 @@
         <v>30</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H32" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="31">
+    <row r="33" spans="1:8">
       <c r="A33" s="21" t="s">
-        <v>203</v>
+        <v>269</v>
       </c>
       <c r="C33" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D33" t="s">
         <v>126</v>
@@ -6137,18 +6542,18 @@
         <v>30</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H33" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" ht="31">
       <c r="A34" s="8" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C34" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D34" t="s">
         <v>126</v>
@@ -6157,18 +6562,18 @@
         <v>30</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H34" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="31">
+    <row r="35" spans="1:8">
       <c r="A35" s="8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C35" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D35" t="s">
         <v>126</v>
@@ -6177,18 +6582,18 @@
         <v>30</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H35" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" ht="31">
       <c r="A36" s="8" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C36" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D36" t="s">
         <v>126</v>
@@ -6197,7 +6602,7 @@
         <v>30</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H36" t="s">
         <v>125</v>
@@ -6205,10 +6610,10 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="8" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C37" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D37" t="s">
         <v>126</v>
@@ -6217,9 +6622,89 @@
         <v>30</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H37" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" t="s">
+        <v>245</v>
+      </c>
+      <c r="D38" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="12">
+        <v>30</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H38" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="C39" t="s">
+        <v>245</v>
+      </c>
+      <c r="D39" t="s">
+        <v>126</v>
+      </c>
+      <c r="E39" s="12">
+        <v>30</v>
+      </c>
+      <c r="G39" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H39" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C40" t="s">
+        <v>245</v>
+      </c>
+      <c r="D40" t="s">
+        <v>126</v>
+      </c>
+      <c r="E40" s="12">
+        <v>30</v>
+      </c>
+      <c r="G40" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H40" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="C41" t="s">
+        <v>245</v>
+      </c>
+      <c r="D41" t="s">
+        <v>126</v>
+      </c>
+      <c r="E41" s="12">
+        <v>30</v>
+      </c>
+      <c r="G41" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="H41" t="s">
         <v>125</v>
       </c>
     </row>
@@ -6231,10 +6716,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC2276F-B0B8-6047-8DEC-2FD310B59F97}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="69.08203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="66.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.5" bestFit="1" customWidth="1"/>
@@ -6263,10 +6748,10 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H1" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="77.5">
@@ -6274,7 +6759,7 @@
         <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D2" t="s">
         <v>126</v>
@@ -6283,7 +6768,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H2" t="s">
         <v>61</v>
@@ -6294,7 +6779,7 @@
         <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D3" t="s">
         <v>126</v>
@@ -6303,7 +6788,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H3" t="s">
         <v>61</v>
@@ -6314,7 +6799,7 @@
         <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D4" t="s">
         <v>126</v>
@@ -6323,7 +6808,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H4" t="s">
         <v>61</v>
@@ -6334,7 +6819,7 @@
         <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D5" t="s">
         <v>126</v>
@@ -6343,7 +6828,7 @@
         <v>30</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
@@ -6354,7 +6839,7 @@
         <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D6" t="s">
         <v>126</v>
@@ -6363,7 +6848,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H6" t="s">
         <v>61</v>
@@ -6374,7 +6859,7 @@
         <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D7" t="s">
         <v>126</v>
@@ -6383,7 +6868,7 @@
         <v>60</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H7" t="s">
         <v>61</v>
@@ -6394,7 +6879,7 @@
         <v>175</v>
       </c>
       <c r="C8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D8" t="s">
         <v>126</v>
@@ -6403,7 +6888,7 @@
         <v>30</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H8" t="s">
         <v>61</v>
@@ -6414,7 +6899,7 @@
         <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D9" t="s">
         <v>126</v>
@@ -6423,7 +6908,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H9" t="s">
         <v>61</v>
@@ -6434,7 +6919,7 @@
         <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D10" t="s">
         <v>126</v>
@@ -6443,7 +6928,7 @@
         <v>30</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H10" t="s">
         <v>61</v>
@@ -6454,7 +6939,7 @@
         <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D11" t="s">
         <v>126</v>
@@ -6463,7 +6948,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H11" t="s">
         <v>61</v>
@@ -6471,50 +6956,50 @@
     </row>
     <row r="12" spans="1:8" ht="77.5">
       <c r="A12" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="C12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="12">
+        <v>30</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="77.5">
+      <c r="A13" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E13" s="12">
+        <v>30</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="93">
+      <c r="A14" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="C12" t="s">
-        <v>249</v>
-      </c>
-      <c r="D12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="12">
-        <v>30</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="H12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="93">
-      <c r="A13" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" t="s">
-        <v>249</v>
-      </c>
-      <c r="D13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E13" s="12">
-        <v>30</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="H13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="77.5">
-      <c r="A14" s="21" t="s">
-        <v>181</v>
-      </c>
       <c r="C14" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D14" t="s">
         <v>126</v>
@@ -6523,7 +7008,7 @@
         <v>50</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H14" t="s">
         <v>61</v>
@@ -6531,10 +7016,10 @@
     </row>
     <row r="15" spans="1:8" ht="77.5">
       <c r="A15" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C15" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D15" t="s">
         <v>126</v>
@@ -6543,7 +7028,7 @@
         <v>50</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H15" t="s">
         <v>61</v>
@@ -6551,10 +7036,10 @@
     </row>
     <row r="16" spans="1:8" ht="77.5">
       <c r="A16" s="21" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D16" t="s">
         <v>126</v>
@@ -6563,18 +7048,18 @@
         <v>50</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="62">
+    <row r="17" spans="1:8" ht="77.5">
       <c r="A17" s="21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D17" t="s">
         <v>126</v>
@@ -6583,18 +7068,18 @@
         <v>0</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H17" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="93">
+    <row r="18" spans="1:8" ht="62">
       <c r="A18" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C18" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D18" t="s">
         <v>126</v>
@@ -6603,7 +7088,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H18" t="s">
         <v>61</v>
@@ -6611,10 +7096,10 @@
     </row>
     <row r="19" spans="1:8" ht="93">
       <c r="A19" s="21" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C19" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D19" t="s">
         <v>126</v>
@@ -6623,18 +7108,18 @@
         <v>50</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="108.5">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="93">
       <c r="A20" s="21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C20" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D20" t="s">
         <v>126</v>
@@ -6643,18 +7128,18 @@
         <v>50</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="93">
+    <row r="21" spans="1:8" ht="108.5">
       <c r="A21" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C21" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D21" t="s">
         <v>126</v>
@@ -6663,7 +7148,7 @@
         <v>30</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H21" t="s">
         <v>124</v>
@@ -6671,10 +7156,10 @@
     </row>
     <row r="22" spans="1:8" ht="93">
       <c r="A22" s="21" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C22" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D22" t="s">
         <v>126</v>
@@ -6683,18 +7168,18 @@
         <v>30</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H22" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="108.5">
+    <row r="23" spans="1:8" ht="93">
       <c r="A23" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C23" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D23" t="s">
         <v>126</v>
@@ -6703,18 +7188,18 @@
         <v>60</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="93">
+    <row r="24" spans="1:8" ht="108.5">
       <c r="A24" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C24" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -6723,18 +7208,18 @@
         <v>60</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="62">
+    <row r="25" spans="1:8" ht="93">
       <c r="A25" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C25" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D25" t="s">
         <v>126</v>
@@ -6743,18 +7228,18 @@
         <v>50</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H25" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="77.5">
+    <row r="26" spans="1:8" ht="62">
       <c r="A26" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C26" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D26" t="s">
         <v>126</v>
@@ -6763,18 +7248,18 @@
         <v>50</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H26" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="93">
+    <row r="27" spans="1:8" ht="77.5">
       <c r="A27" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D27" t="s">
         <v>126</v>
@@ -6783,18 +7268,18 @@
         <v>40</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="93">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="77.5">
       <c r="A28" s="8" t="s">
-        <v>198</v>
+        <v>252</v>
       </c>
       <c r="C28" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D28" t="s">
         <v>126</v>
@@ -6803,18 +7288,18 @@
         <v>40</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H28" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="77.5">
+    <row r="29" spans="1:8" ht="93">
       <c r="A29" s="21" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D29" t="s">
         <v>126</v>
@@ -6823,7 +7308,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H29" t="s">
         <v>125</v>
@@ -6831,10 +7316,10 @@
     </row>
     <row r="30" spans="1:8" ht="62">
       <c r="A30" s="21" t="s">
-        <v>200</v>
+        <v>253</v>
       </c>
       <c r="C30" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D30" t="s">
         <v>126</v>
@@ -6843,18 +7328,18 @@
         <v>40</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H30" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="77.5">
+    <row r="31" spans="1:8" ht="62">
       <c r="A31" s="21" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C31" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D31" t="s">
         <v>126</v>
@@ -6863,7 +7348,7 @@
         <v>30</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H31" t="s">
         <v>125</v>
@@ -6871,10 +7356,10 @@
     </row>
     <row r="32" spans="1:8" ht="62">
       <c r="A32" s="21" t="s">
-        <v>202</v>
+        <v>268</v>
       </c>
       <c r="C32" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D32" t="s">
         <v>126</v>
@@ -6883,18 +7368,18 @@
         <v>30</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H32" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="77.5">
+    <row r="33" spans="1:8" ht="62">
       <c r="A33" s="21" t="s">
-        <v>203</v>
+        <v>269</v>
       </c>
       <c r="C33" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D33" t="s">
         <v>126</v>
@@ -6903,18 +7388,18 @@
         <v>30</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H33" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="62">
+    <row r="34" spans="1:8" ht="77.5">
       <c r="A34" s="8" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C34" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D34" t="s">
         <v>126</v>
@@ -6923,38 +7408,38 @@
         <v>30</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H34" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="77.5">
+    <row r="35" spans="1:8" ht="62">
       <c r="A35" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C35" t="s">
+        <v>246</v>
+      </c>
+      <c r="D35" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="12">
+        <v>30</v>
+      </c>
+      <c r="G35" s="12" t="s">
         <v>205</v>
-      </c>
-      <c r="C35" t="s">
-        <v>249</v>
-      </c>
-      <c r="D35" t="s">
-        <v>126</v>
-      </c>
-      <c r="E35" s="12">
-        <v>30</v>
-      </c>
-      <c r="G35" s="12" t="s">
-        <v>208</v>
       </c>
       <c r="H35" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="46.5">
+    <row r="36" spans="1:8" ht="77.5">
       <c r="A36" s="8" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C36" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D36" t="s">
         <v>126</v>
@@ -6963,7 +7448,7 @@
         <v>30</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H36" t="s">
         <v>125</v>
@@ -6971,10 +7456,10 @@
     </row>
     <row r="37" spans="1:8" ht="62">
       <c r="A37" s="8" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C37" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D37" t="s">
         <v>126</v>
@@ -6983,22 +7468,104 @@
         <v>30</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H37" t="s">
         <v>125</v>
       </c>
     </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" t="s">
+        <v>246</v>
+      </c>
+      <c r="D38" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="12">
+        <v>30</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H38" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="C39" t="s">
+        <v>246</v>
+      </c>
+      <c r="D39" t="s">
+        <v>126</v>
+      </c>
+      <c r="E39" s="12">
+        <v>30</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H39" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C40" t="s">
+        <v>246</v>
+      </c>
+      <c r="D40" t="s">
+        <v>126</v>
+      </c>
+      <c r="E40" s="12">
+        <v>30</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H40" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="C41" t="s">
+        <v>246</v>
+      </c>
+      <c r="D41" t="s">
+        <v>126</v>
+      </c>
+      <c r="E41" s="12">
+        <v>30</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="H41" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{125867D4-4268-FD46-BD8D-BFA58B4600F1}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5"/>
   <cols>
+    <col min="1" max="1" width="69.08203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="24.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -7024,10 +7591,10 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H1" s="22" t="s">
         <v>186</v>
-      </c>
-      <c r="H1" s="22" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="170.5">
@@ -7035,7 +7602,7 @@
         <v>169</v>
       </c>
       <c r="C2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D2" t="s">
         <v>126</v>
@@ -7044,7 +7611,7 @@
         <v>30</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H2" t="s">
         <v>61</v>
@@ -7055,7 +7622,7 @@
         <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D3" t="s">
         <v>126</v>
@@ -7064,7 +7631,7 @@
         <v>30</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H3" t="s">
         <v>61</v>
@@ -7075,7 +7642,7 @@
         <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D4" t="s">
         <v>126</v>
@@ -7084,7 +7651,7 @@
         <v>30</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H4" t="s">
         <v>61</v>
@@ -7095,7 +7662,7 @@
         <v>172</v>
       </c>
       <c r="C5" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D5" t="s">
         <v>126</v>
@@ -7104,7 +7671,7 @@
         <v>30</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H5" t="s">
         <v>61</v>
@@ -7115,7 +7682,7 @@
         <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D6" t="s">
         <v>126</v>
@@ -7124,7 +7691,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H6" t="s">
         <v>61</v>
@@ -7135,7 +7702,7 @@
         <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D7" t="s">
         <v>126</v>
@@ -7144,7 +7711,7 @@
         <v>60</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H7" t="s">
         <v>61</v>
@@ -7155,7 +7722,7 @@
         <v>175</v>
       </c>
       <c r="C8" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D8" t="s">
         <v>126</v>
@@ -7164,7 +7731,7 @@
         <v>30</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H8" t="s">
         <v>61</v>
@@ -7175,7 +7742,7 @@
         <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D9" t="s">
         <v>126</v>
@@ -7184,7 +7751,7 @@
         <v>30</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H9" t="s">
         <v>61</v>
@@ -7195,7 +7762,7 @@
         <v>177</v>
       </c>
       <c r="C10" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D10" t="s">
         <v>126</v>
@@ -7204,7 +7771,7 @@
         <v>30</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H10" t="s">
         <v>61</v>
@@ -7215,7 +7782,7 @@
         <v>178</v>
       </c>
       <c r="C11" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D11" t="s">
         <v>126</v>
@@ -7224,7 +7791,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H11" t="s">
         <v>61</v>
@@ -7232,50 +7799,50 @@
     </row>
     <row r="12" spans="1:8" ht="124">
       <c r="A12" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="C12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E12" s="12">
+        <v>30</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="124">
+      <c r="A13" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="C13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E13" s="12">
+        <v>30</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="170.5">
+      <c r="A14" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="C12" t="s">
-        <v>249</v>
-      </c>
-      <c r="D12" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="12">
-        <v>30</v>
-      </c>
-      <c r="G12" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="H12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="170.5">
-      <c r="A13" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" t="s">
-        <v>249</v>
-      </c>
-      <c r="D13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E13" s="12">
-        <v>30</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>209</v>
-      </c>
-      <c r="H13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="155">
-      <c r="A14" s="21" t="s">
-        <v>181</v>
-      </c>
       <c r="C14" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D14" t="s">
         <v>126</v>
@@ -7284,18 +7851,18 @@
         <v>50</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H14" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="139.5">
+    <row r="15" spans="1:8" ht="155">
       <c r="A15" s="21" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C15" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D15" t="s">
         <v>126</v>
@@ -7304,18 +7871,18 @@
         <v>50</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="155">
+    <row r="16" spans="1:8" ht="139.5">
       <c r="A16" s="21" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D16" t="s">
         <v>126</v>
@@ -7324,18 +7891,18 @@
         <v>50</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="93">
+    <row r="17" spans="1:8" ht="155">
       <c r="A17" s="21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D17" t="s">
         <v>126</v>
@@ -7344,18 +7911,18 @@
         <v>0</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H17" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="186">
+    <row r="18" spans="1:8" ht="93">
       <c r="A18" s="21" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C18" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D18" t="s">
         <v>126</v>
@@ -7364,18 +7931,18 @@
         <v>0</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H18" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="155">
+    <row r="19" spans="1:8" ht="186">
       <c r="A19" s="21" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C19" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D19" t="s">
         <v>126</v>
@@ -7384,18 +7951,18 @@
         <v>50</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="186">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="155">
       <c r="A20" s="21" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C20" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D20" t="s">
         <v>126</v>
@@ -7404,7 +7971,7 @@
         <v>50</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
@@ -7412,10 +7979,10 @@
     </row>
     <row r="21" spans="1:8" ht="186">
       <c r="A21" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C21" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D21" t="s">
         <v>126</v>
@@ -7424,18 +7991,18 @@
         <v>30</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H21" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="139.5">
+    <row r="22" spans="1:8" ht="186">
       <c r="A22" s="21" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C22" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D22" t="s">
         <v>126</v>
@@ -7444,18 +8011,18 @@
         <v>30</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H22" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="217">
+    <row r="23" spans="1:8" ht="139.5">
       <c r="A23" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C23" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D23" t="s">
         <v>126</v>
@@ -7464,18 +8031,18 @@
         <v>60</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H23" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="170.5">
+    <row r="24" spans="1:8" ht="217">
       <c r="A24" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C24" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D24" t="s">
         <v>126</v>
@@ -7484,18 +8051,18 @@
         <v>60</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H24" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="124">
+    <row r="25" spans="1:8" ht="170.5">
       <c r="A25" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C25" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D25" t="s">
         <v>126</v>
@@ -7504,18 +8071,18 @@
         <v>50</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H25" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="155">
+    <row r="26" spans="1:8" ht="124">
       <c r="A26" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C26" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D26" t="s">
         <v>126</v>
@@ -7524,18 +8091,18 @@
         <v>50</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H26" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="139.5">
+    <row r="27" spans="1:8" ht="155">
       <c r="A27" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D27" t="s">
         <v>126</v>
@@ -7544,18 +8111,18 @@
         <v>40</v>
       </c>
       <c r="G27" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="170.5">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="139.5">
       <c r="A28" s="8" t="s">
-        <v>198</v>
+        <v>252</v>
       </c>
       <c r="C28" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D28" t="s">
         <v>126</v>
@@ -7564,18 +8131,18 @@
         <v>40</v>
       </c>
       <c r="G28" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H28" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="139.5">
+    <row r="29" spans="1:8" ht="170.5">
       <c r="A29" s="21" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C29" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D29" t="s">
         <v>126</v>
@@ -7584,18 +8151,18 @@
         <v>40</v>
       </c>
       <c r="G29" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H29" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="124">
+    <row r="30" spans="1:8" ht="139.5">
       <c r="A30" s="21" t="s">
-        <v>200</v>
+        <v>253</v>
       </c>
       <c r="C30" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D30" t="s">
         <v>126</v>
@@ -7604,18 +8171,18 @@
         <v>40</v>
       </c>
       <c r="G30" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H30" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="155">
+    <row r="31" spans="1:8" ht="124">
       <c r="A31" s="21" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C31" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D31" t="s">
         <v>126</v>
@@ -7624,7 +8191,7 @@
         <v>30</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H31" t="s">
         <v>125</v>
@@ -7632,10 +8199,10 @@
     </row>
     <row r="32" spans="1:8" ht="124">
       <c r="A32" s="21" t="s">
-        <v>202</v>
+        <v>268</v>
       </c>
       <c r="C32" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D32" t="s">
         <v>126</v>
@@ -7644,18 +8211,18 @@
         <v>30</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H32" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="139.5">
+    <row r="33" spans="1:8" ht="108.5">
       <c r="A33" s="21" t="s">
-        <v>203</v>
+        <v>269</v>
       </c>
       <c r="C33" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D33" t="s">
         <v>126</v>
@@ -7664,18 +8231,18 @@
         <v>30</v>
       </c>
       <c r="G33" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H33" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="124">
+    <row r="34" spans="1:8" ht="155">
       <c r="A34" s="8" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C34" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D34" t="s">
         <v>126</v>
@@ -7684,18 +8251,18 @@
         <v>30</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H34" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="139.5">
+    <row r="35" spans="1:8" ht="124">
       <c r="A35" s="8" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C35" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D35" t="s">
         <v>126</v>
@@ -7704,27 +8271,27 @@
         <v>30</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H35" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="108.5">
+    <row r="36" spans="1:8" ht="139.5">
       <c r="A36" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C36" t="s">
+        <v>246</v>
+      </c>
+      <c r="D36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E36" s="12">
+        <v>30</v>
+      </c>
+      <c r="G36" s="20" t="s">
         <v>206</v>
-      </c>
-      <c r="C36" t="s">
-        <v>249</v>
-      </c>
-      <c r="D36" t="s">
-        <v>126</v>
-      </c>
-      <c r="E36" s="12">
-        <v>30</v>
-      </c>
-      <c r="G36" s="20" t="s">
-        <v>209</v>
       </c>
       <c r="H36" t="s">
         <v>125</v>
@@ -7732,10 +8299,10 @@
     </row>
     <row r="37" spans="1:8" ht="124">
       <c r="A37" s="8" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C37" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D37" t="s">
         <v>126</v>
@@ -7744,9 +8311,89 @@
         <v>30</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H37" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" t="s">
+        <v>246</v>
+      </c>
+      <c r="D38" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="12">
+        <v>30</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H38" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="C39" t="s">
+        <v>246</v>
+      </c>
+      <c r="D39" t="s">
+        <v>126</v>
+      </c>
+      <c r="E39" s="12">
+        <v>30</v>
+      </c>
+      <c r="G39" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H39" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="C40" t="s">
+        <v>246</v>
+      </c>
+      <c r="D40" t="s">
+        <v>126</v>
+      </c>
+      <c r="E40" s="12">
+        <v>30</v>
+      </c>
+      <c r="G40" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H40" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="C41" t="s">
+        <v>246</v>
+      </c>
+      <c r="D41" t="s">
+        <v>126</v>
+      </c>
+      <c r="E41" s="12">
+        <v>30</v>
+      </c>
+      <c r="G41" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="H41" t="s">
         <v>125</v>
       </c>
     </row>

</xml_diff>